<commit_message>
Update posts.xlsx after post
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C809"/>
+  <dimension ref="A1:C808"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14189,28 +14189,6 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t xml:space="preserve">「諸行無常」كلّ شيءٍ يتغيّر
-クッル・シャイイン・ヤタガイヤル [kullu Shay'in ya-taGhayyaru]
-「あらゆる物は」[kullu Shay'in]・「それは変わる」[ya-taGhayyaru] 
-諸行無常（ショギョウ・ムジョウ）
-2510 
-د. ماجد عبدالله </t>
-        </is>
-      </c>
-      <c r="B654" t="inlineStr">
-        <is>
-          <t>images/「諸行無常」_img1.jpg</t>
-        </is>
-      </c>
-      <c r="C654" t="inlineStr">
-        <is>
-          <t>表紙 ,タイトル</t>
-        </is>
-      </c>
-    </row>
-    <row r="655">
-      <c r="A655" t="inlineStr">
-        <is>
           <t xml:space="preserve">「幸せな人生には弱い記憶力が必要」
 الحياة السعيدة تتطلب ذاكرة ضعيفة
 [al-Hayaatu ^sa*iidatu ta-ta_tallabu Dhaakiratan _da*iifatan]
@@ -14218,19 +14196,19 @@
 2012 出典不明 </t>
         </is>
       </c>
-      <c r="B655" t="inlineStr">
+      <c r="B654" t="inlineStr">
         <is>
           <t>images/「幸せな人生には弱い記憶力が必要」_img1.jpg</t>
         </is>
       </c>
-      <c r="C655" t="inlineStr">
+      <c r="C654" t="inlineStr">
         <is>
           <t>前向き</t>
         </is>
       </c>
     </row>
-    <row r="656">
-      <c r="A656" t="inlineStr">
+    <row r="655">
+      <c r="A655" t="inlineStr">
         <is>
           <t xml:space="preserve">「このパンダは私たちに、幸せは単純なことの中に隠れているのだと教えている」
 دب "الباندا" هذا يؤكد لنا أن السعادة تكمن في أبسط الأشياء
@@ -14238,19 +14216,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1309938472065486848 </t>
         </is>
       </c>
-      <c r="B656" t="inlineStr">
+      <c r="B655" t="inlineStr">
         <is>
           <t>images/「このパンダは私たちに、幸せは単純なこ.png</t>
         </is>
       </c>
-      <c r="C656" t="inlineStr">
+      <c r="C655" t="inlineStr">
         <is>
           <t>パンダ ,雪</t>
         </is>
       </c>
     </row>
-    <row r="657">
-      <c r="A657" t="inlineStr">
+    <row r="656">
+      <c r="A656" t="inlineStr">
         <is>
           <t xml:space="preserve">「良い時間は速く過ぎる」
 الأوقات الجميلة تمر بسرعة
@@ -14260,19 +14238,19 @@
 1810 Nasser.Tumblr </t>
         </is>
       </c>
-      <c r="B657" t="inlineStr">
+      <c r="B656" t="inlineStr">
         <is>
           <t>images/「良い時間は速く過ぎる」_img1.jpg</t>
         </is>
       </c>
-      <c r="C657" t="inlineStr">
+      <c r="C656" t="inlineStr">
         <is>
           <t>相対論 ,心理学</t>
         </is>
       </c>
     </row>
-    <row r="658">
-      <c r="A658" t="inlineStr">
+    <row r="657">
+      <c r="A657" t="inlineStr">
         <is>
           <t xml:space="preserve">「今日が始まりかもしれない」
 كل يوم ممكن يكون بداية
@@ -14282,19 +14260,19 @@
 2308 Ahmed Madyan </t>
         </is>
       </c>
-      <c r="B658" t="inlineStr">
+      <c r="B657" t="inlineStr">
         <is>
           <t>images/「今日が始まりかもしれない」_img1.jpg</t>
         </is>
       </c>
-      <c r="C658" t="inlineStr">
+      <c r="C657" t="inlineStr">
         <is>
           <t>吉日 ,開始</t>
         </is>
       </c>
     </row>
-    <row r="659">
-      <c r="A659" t="inlineStr">
+    <row r="658">
+      <c r="A658" t="inlineStr">
         <is>
           <t xml:space="preserve">「ヌール、歯医者さんに行く」
 نور تذهب إلى طبيب الأسنان
@@ -14304,19 +14282,19 @@
 2109 RABIE </t>
         </is>
       </c>
-      <c r="B659" t="inlineStr">
+      <c r="B658" t="inlineStr">
         <is>
           <t>images/「ヌール、歯医者さんに行く」_img1.jpg</t>
         </is>
       </c>
-      <c r="C659" t="inlineStr">
+      <c r="C658" t="inlineStr">
         <is>
           <t>絵本 ,歯科</t>
         </is>
       </c>
     </row>
-    <row r="660">
-      <c r="A660" t="inlineStr">
+    <row r="659">
+      <c r="A659" t="inlineStr">
         <is>
           <t xml:space="preserve">「ラヤンはねむれない」
 لَيان لا تَسْتَطيعُ أَنْ تَنام
@@ -14325,19 +14303,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B660" t="inlineStr">
+      <c r="B659" t="inlineStr">
         <is>
           <t>images/「ラヤンはねむれない」_img1.jpg</t>
         </is>
       </c>
-      <c r="C660" t="inlineStr">
+      <c r="C659" t="inlineStr">
         <is>
           <t>絵本 ,不眠症</t>
         </is>
       </c>
     </row>
-    <row r="661">
-      <c r="A661" t="inlineStr">
+    <row r="660">
+      <c r="A660" t="inlineStr">
         <is>
           <t xml:space="preserve">「クネイトラ県、蜂の巣を約60%失う」
 القنيطرة تفقد حوالي 60 % من خلايا نحلها
@@ -14345,19 +14323,19 @@
 2403 nabd com/t/101679025-fb119f </t>
         </is>
       </c>
-      <c r="B661" t="inlineStr">
+      <c r="B660" t="inlineStr">
         <is>
           <t>images/「クネイトラ県、蜂の巣を約60%失う」_img1.jpg</t>
         </is>
       </c>
-      <c r="C661" t="inlineStr">
+      <c r="C660" t="inlineStr">
         <is>
           <t>蜂の巣 ,パーセント</t>
         </is>
       </c>
     </row>
-    <row r="662">
-      <c r="A662" t="inlineStr">
+    <row r="661">
+      <c r="A661" t="inlineStr">
         <is>
           <t xml:space="preserve">「結ばれしター」ة
 ⁦( تاء مربوطة )[taa' marbuu_ta]：ت「ター」( تاء )[taa']・「結ばれている」( مربوط )[marbuu_t]：( ربط )【結】⁩
@@ -14365,19 +14343,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B662" t="inlineStr">
+      <c r="B661" t="inlineStr">
         <is>
           <t>images/「結ばれしター」_img1.jpg</t>
         </is>
       </c>
-      <c r="C662" t="inlineStr">
+      <c r="C661" t="inlineStr">
         <is>
           <t>アラビア文字 ,顔</t>
         </is>
       </c>
     </row>
-    <row r="663">
-      <c r="A663" t="inlineStr">
+    <row r="662">
+      <c r="A662" t="inlineStr">
         <is>
           <t xml:space="preserve">「忙しい」مشغول
 マシュグール [maShGhuul]
@@ -14386,19 +14364,19 @@
 1811 skyshinichi.instagram </t>
         </is>
       </c>
-      <c r="B663" t="inlineStr">
+      <c r="B662" t="inlineStr">
         <is>
           <t>images/「忙しい」_img1.jpg</t>
         </is>
       </c>
-      <c r="C663" t="inlineStr">
+      <c r="C662" t="inlineStr">
         <is>
           <t>スティッチ ,残業</t>
         </is>
       </c>
     </row>
-    <row r="664">
-      <c r="A664" t="inlineStr">
+    <row r="663">
+      <c r="A663" t="inlineStr">
         <is>
           <t xml:space="preserve">「駐車禁止」ممنوع الوقوف
 マムヌーア・アルウクーフ [mamnuu* al-wuquuf]
@@ -14407,19 +14385,19 @@
 2106 出典不明 </t>
         </is>
       </c>
-      <c r="B664" t="inlineStr">
+      <c r="B663" t="inlineStr">
         <is>
           <t>images/「駐車禁止」_img1.jpg</t>
         </is>
       </c>
-      <c r="C664" t="inlineStr">
+      <c r="C663" t="inlineStr">
         <is>
           <t>標識 ,ジョーク</t>
         </is>
       </c>
     </row>
-    <row r="665">
-      <c r="A665" t="inlineStr">
+    <row r="664">
+      <c r="A664" t="inlineStr">
         <is>
           <t xml:space="preserve">「一人ひとりが責任を」
 كُلنا مسؤول
@@ -14429,19 +14407,19 @@
 2308 covid19awareness sa </t>
         </is>
       </c>
-      <c r="B665" t="inlineStr">
+      <c r="B664" t="inlineStr">
         <is>
           <t>images/「一人ひとりが責任を」_img1.jpg</t>
         </is>
       </c>
-      <c r="C665" t="inlineStr">
+      <c r="C664" t="inlineStr">
         <is>
           <t>Covid ,感染拡大防止</t>
         </is>
       </c>
     </row>
-    <row r="666">
-      <c r="A666" t="inlineStr">
+    <row r="665">
+      <c r="A665" t="inlineStr">
         <is>
           <t xml:space="preserve">「おめでとうございます」مبروك
 マブルーク [mabruuk]
@@ -14450,19 +14428,19 @@
 2308 </t>
         </is>
       </c>
-      <c r="B666" t="inlineStr">
+      <c r="B665" t="inlineStr">
         <is>
           <t>images/「おめでとうございます」_img1.jpg</t>
         </is>
       </c>
-      <c r="C666" t="inlineStr">
+      <c r="C665" t="inlineStr">
         <is>
           <t>詐欺 ,広告</t>
         </is>
       </c>
     </row>
-    <row r="667">
-      <c r="A667" t="inlineStr">
+    <row r="666">
+      <c r="A666" t="inlineStr">
         <is>
           <t xml:space="preserve">「手書きフォント」
 خط مكتوب باليد
@@ -14472,19 +14450,19 @@
 1809 FahdAlFraikh Behance </t>
         </is>
       </c>
-      <c r="B667" t="inlineStr">
+      <c r="B666" t="inlineStr">
         <is>
           <t>images/「手書きフォント」_img1.jpg</t>
         </is>
       </c>
-      <c r="C667" t="inlineStr">
+      <c r="C666" t="inlineStr">
         <is>
           <t>可愛いフォント ,筆跡</t>
         </is>
       </c>
     </row>
-    <row r="668">
-      <c r="A668" t="inlineStr">
+    <row r="667">
+      <c r="A667" t="inlineStr">
         <is>
           <t xml:space="preserve">「開かれたターと結ばれたター」
 التاء المفتوحة والمربوطة
@@ -14494,19 +14472,19 @@
 2109 slideshare.net </t>
         </is>
       </c>
-      <c r="B668" t="inlineStr">
+      <c r="B667" t="inlineStr">
         <is>
           <t>images/「開かれたターと結ばれたター」_img1.jpg</t>
         </is>
       </c>
-      <c r="C668" t="inlineStr">
+      <c r="C667" t="inlineStr">
         <is>
           <t>アラビア文字 ,スマイリー</t>
         </is>
       </c>
     </row>
-    <row r="669">
-      <c r="A669" t="inlineStr">
+    <row r="668">
+      <c r="A668" t="inlineStr">
         <is>
           <t xml:space="preserve">「このラマは誇らしげにして立っている」
 تقف هذه اللاما مزهوة بنفسها
@@ -14514,19 +14492,19 @@
 2410 https://twitter.com/NatGeoMagArab/status/1597485552965935104 </t>
         </is>
       </c>
-      <c r="B669" t="inlineStr">
+      <c r="B668" t="inlineStr">
         <is>
           <t>images/「このラマは誇らしげにして立っている」_img1.jpg</t>
         </is>
       </c>
-      <c r="C669" t="inlineStr">
+      <c r="C668" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,マチュピチュ遺跡</t>
         </is>
       </c>
     </row>
-    <row r="670">
-      <c r="A670" t="inlineStr">
+    <row r="669">
+      <c r="A669" t="inlineStr">
         <is>
           <t xml:space="preserve">「小さな生き物にしては危険な名前だ」
 اسم خطير لمخلوق صغير
@@ -14535,19 +14513,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1495035772071669760 </t>
         </is>
       </c>
-      <c r="B670" t="inlineStr">
+      <c r="B669" t="inlineStr">
         <is>
           <t>images/「小さな生き物にしては危険な名前だ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C670" t="inlineStr">
+      <c r="C669" t="inlineStr">
         <is>
           <t>有袋類 ,タスマニアデビル</t>
         </is>
       </c>
     </row>
-    <row r="671">
-      <c r="A671" t="inlineStr">
+    <row r="670">
+      <c r="A670" t="inlineStr">
         <is>
           <t xml:space="preserve">「こわれている」مكسر
 ムカッサル [mukassar]
@@ -14555,19 +14533,19 @@
 2105 behance Written-Visuals </t>
         </is>
       </c>
-      <c r="B671" t="inlineStr">
+      <c r="B670" t="inlineStr">
         <is>
           <t>images/「こわれている」_img1.jpg</t>
         </is>
       </c>
-      <c r="C671" t="inlineStr">
+      <c r="C670" t="inlineStr">
         <is>
           <t>バラバラ ,デザイン</t>
         </is>
       </c>
     </row>
-    <row r="672">
-      <c r="A672" t="inlineStr">
+    <row r="671">
+      <c r="A671" t="inlineStr">
         <is>
           <t xml:space="preserve">「早起きする方法」
 كيف تنهض مُبكّرًا
@@ -14577,19 +14555,19 @@
 2308 Funders and Founders </t>
         </is>
       </c>
-      <c r="B672" t="inlineStr">
+      <c r="B671" t="inlineStr">
         <is>
           <t>images/「早起きする方法」_img1.jpg</t>
         </is>
       </c>
-      <c r="C672" t="inlineStr">
+      <c r="C671" t="inlineStr">
         <is>
           <t>オフトゥン ,寝起き</t>
         </is>
       </c>
     </row>
-    <row r="673">
-      <c r="A673" t="inlineStr">
+    <row r="672">
+      <c r="A672" t="inlineStr">
         <is>
           <t xml:space="preserve">「アラブ・デザイン文字展覧会」
 معرض لتخطيط الحرف العربي
@@ -14599,38 +14577,38 @@
 2109 arabic lettering exhibition </t>
         </is>
       </c>
-      <c r="B673" t="inlineStr">
+      <c r="B672" t="inlineStr">
         <is>
           <t>images/「アラブ・デザイン文字展覧会」_img1.jpg</t>
         </is>
       </c>
-      <c r="C673" t="inlineStr">
+      <c r="C672" t="inlineStr">
         <is>
           <t>ポスター</t>
         </is>
       </c>
     </row>
-    <row r="674">
-      <c r="A674" t="inlineStr">
+    <row r="673">
+      <c r="A673" t="inlineStr">
         <is>
           <t xml:space="preserve">「お気に入りのおもちゃには触らせない」
 ⁦「彼は〜を許さない」[laa ya-smaHu bi-]：「彼は許す」( يسمح )[ya-smaH(u)]：「許した」( سمح )[samaHa]：( سَ )[sa]・( مَ )[ma]・( حَ )[Ha]⁩
 2209 https://pic.twitter.com/qWcIPB3fz2 </t>
         </is>
       </c>
-      <c r="B674" t="inlineStr">
+      <c r="B673" t="inlineStr">
         <is>
           <t>images/「お気に入りのおもちゃには触らせない」_img1.jpg</t>
         </is>
       </c>
-      <c r="C674" t="inlineStr">
+      <c r="C673" t="inlineStr">
         <is>
           <t>パンダ ,ボール</t>
         </is>
       </c>
     </row>
-    <row r="675">
-      <c r="A675" t="inlineStr">
+    <row r="674">
+      <c r="A674" t="inlineStr">
         <is>
           <t xml:space="preserve">「名探偵コナン」المحقق كونان
 アルムハッキク・コナン [al-muHaqqiq Conan]
@@ -14639,19 +14617,19 @@
 1809 wikipedia </t>
         </is>
       </c>
-      <c r="B675" t="inlineStr">
+      <c r="B674" t="inlineStr">
         <is>
           <t>images/「名探偵コナン」_img1.jpg</t>
         </is>
       </c>
-      <c r="C675" t="inlineStr">
+      <c r="C674" t="inlineStr">
         <is>
           <t>江戸川コナン ,ロゴ</t>
         </is>
       </c>
     </row>
-    <row r="676">
-      <c r="A676" t="inlineStr">
+    <row r="675">
+      <c r="A675" t="inlineStr">
         <is>
           <t xml:space="preserve">「イードおめでとう」عيد مبارك
 イード・ムバーラク [*iid mubaarak]
@@ -14659,19 +14637,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B676" t="inlineStr">
+      <c r="B675" t="inlineStr">
         <is>
           <t>images/「イードおめでとう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C676" t="inlineStr">
+      <c r="C675" t="inlineStr">
         <is>
           <t>عيد ,アラビア語</t>
         </is>
       </c>
     </row>
-    <row r="677">
-      <c r="A677" t="inlineStr">
+    <row r="676">
+      <c r="A676" t="inlineStr">
         <is>
           <t xml:space="preserve">「戦士」محارب
 ムハーリブ [muHaarib]
@@ -14680,19 +14658,19 @@
 1809 abudinges.tumblr </t>
         </is>
       </c>
-      <c r="B677" t="inlineStr">
+      <c r="B676" t="inlineStr">
         <is>
           <t>images/「戦士」_img1.jpg</t>
         </is>
       </c>
-      <c r="C677" t="inlineStr">
+      <c r="C676" t="inlineStr">
         <is>
           <t>ロゴ ,赤</t>
         </is>
       </c>
     </row>
-    <row r="678">
-      <c r="A678" t="inlineStr">
+    <row r="677">
+      <c r="A677" t="inlineStr">
         <is>
           <t xml:space="preserve">「ライブ」بث مباشر
 バッス・ムバーシル [ba^Th(un) mubaaShir(un)]
@@ -14701,19 +14679,19 @@
 2308 beIN SPORTS </t>
         </is>
       </c>
-      <c r="B678" t="inlineStr">
+      <c r="B677" t="inlineStr">
         <is>
           <t>images/「ライブ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C678" t="inlineStr">
+      <c r="C677" t="inlineStr">
         <is>
           <t xml:space="preserve">生放送 ,試合 </t>
         </is>
       </c>
     </row>
-    <row r="679">
-      <c r="A679" t="inlineStr">
+    <row r="678">
+      <c r="A678" t="inlineStr">
         <is>
           <t xml:space="preserve">「信者」مُؤْمِنٌ
 ムッミン [mu'min(un)]
@@ -14722,19 +14700,19 @@
 2106 出典不明 </t>
         </is>
       </c>
-      <c r="B679" t="inlineStr">
+      <c r="B678" t="inlineStr">
         <is>
           <t>images/「信者」_img1.jpg</t>
         </is>
       </c>
-      <c r="C679" t="inlineStr">
+      <c r="C678" t="inlineStr">
         <is>
           <t>明暗 ,信仰</t>
         </is>
       </c>
     </row>
-    <row r="680">
-      <c r="A680" t="inlineStr">
+    <row r="679">
+      <c r="A679" t="inlineStr">
         <is>
           <t xml:space="preserve">「開⇔閉」
 مفتوح
@@ -14745,19 +14723,19 @@
 2312 Hussein Safina, behance </t>
         </is>
       </c>
-      <c r="B680" t="inlineStr">
+      <c r="B679" t="inlineStr">
         <is>
           <t>images/「開⇔閉」_img1.jpg</t>
         </is>
       </c>
-      <c r="C680" t="inlineStr">
+      <c r="C679" t="inlineStr">
         <is>
           <t>オープンマインド ,トグル</t>
         </is>
       </c>
     </row>
-    <row r="681">
-      <c r="A681" t="inlineStr">
+    <row r="680">
+      <c r="A680" t="inlineStr">
         <is>
           <t xml:space="preserve">「予想外な結末！」
 نهاية غير متوقعة
@@ -14765,19 +14743,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1159011433444593665 </t>
         </is>
       </c>
-      <c r="B681" t="inlineStr">
+      <c r="B680" t="inlineStr">
         <is>
           <t>images/「予想外な結末！」_img1.jpg</t>
         </is>
       </c>
-      <c r="C681" t="inlineStr">
+      <c r="C680" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,ウサギ</t>
         </is>
       </c>
     </row>
-    <row r="682">
-      <c r="A682" t="inlineStr">
+    <row r="681">
+      <c r="A681" t="inlineStr">
         <is>
           <t xml:space="preserve">「ベイルート・アニメイテッド」
 بیروت متحرّکة
@@ -14787,19 +14765,19 @@
 2308 arabic_script Instagram </t>
         </is>
       </c>
-      <c r="B682" t="inlineStr">
+      <c r="B681" t="inlineStr">
         <is>
           <t>images/「ベイルート・アニメイテッド」_img1.jpg</t>
         </is>
       </c>
-      <c r="C682" t="inlineStr">
+      <c r="C681" t="inlineStr">
         <is>
           <t>アニメ ,レバノン</t>
         </is>
       </c>
     </row>
-    <row r="683">
-      <c r="A683" t="inlineStr">
+    <row r="682">
+      <c r="A682" t="inlineStr">
         <is>
           <t xml:space="preserve">「夢みれば叶う」
 كُلُّ مُتَوَقَّعٍ آتٍ
@@ -14809,19 +14787,19 @@
 2108 Ahmed Madyan </t>
         </is>
       </c>
-      <c r="B683" t="inlineStr">
+      <c r="B682" t="inlineStr">
         <is>
           <t>images/「夢みれば叶う」_img1.jpg</t>
         </is>
       </c>
-      <c r="C683" t="inlineStr">
+      <c r="C682" t="inlineStr">
         <is>
           <t>希望 ,ドリカム</t>
         </is>
       </c>
     </row>
-    <row r="684">
-      <c r="A684" t="inlineStr">
+    <row r="683">
+      <c r="A683" t="inlineStr">
         <is>
           <t xml:space="preserve">「もし両者が人間のように鎧で武装して戦いに突入したら」
 لو خاضا معاركهما متسلحين بالدروع على غرار البش
@@ -14829,19 +14807,19 @@
 2404 https://x.com/NatGeoMagArab/status/1759284149456945464 </t>
         </is>
       </c>
-      <c r="B684" t="inlineStr">
+      <c r="B683" t="inlineStr">
         <is>
           <t>images/「もし両者が人間のように鎧で武装して戦_img1.jpg,images/「もし両者が人間のように鎧で武装して戦_img2.jpg</t>
         </is>
       </c>
-      <c r="C684" t="inlineStr">
+      <c r="C683" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,猫</t>
         </is>
       </c>
     </row>
-    <row r="685">
-      <c r="A685" t="inlineStr">
+    <row r="684">
+      <c r="A684" t="inlineStr">
         <is>
           <t xml:space="preserve">「全ては結びついている」
 كل شيء مترابط
@@ -14851,19 +14829,19 @@
 2308 Ahmed Madyan https://twitter.com/madyco22/status/1451990828298166273 </t>
         </is>
       </c>
-      <c r="B685" t="inlineStr">
+      <c r="B684" t="inlineStr">
         <is>
           <t>images/「全ては結びついている」_img1.jpg</t>
         </is>
       </c>
-      <c r="C685" t="inlineStr">
+      <c r="C684" t="inlineStr">
         <is>
           <t>一筆書き ,デザイン</t>
         </is>
       </c>
     </row>
-    <row r="686">
-      <c r="A686" t="inlineStr">
+    <row r="685">
+      <c r="A685" t="inlineStr">
         <is>
           <t xml:space="preserve">「初心者のためのスケッチトレーニング」
 تعليم الرسم للمبتدئين
@@ -14873,19 +14851,19 @@
 2308 free-bookspdf com </t>
         </is>
       </c>
-      <c r="B686" t="inlineStr">
+      <c r="B685" t="inlineStr">
         <is>
           <t>images/「初心者のためのスケッチトレーニング」_img1.jpg</t>
         </is>
       </c>
-      <c r="C686" t="inlineStr">
+      <c r="C685" t="inlineStr">
         <is>
           <t>イラスト ,絵</t>
         </is>
       </c>
     </row>
-    <row r="687">
-      <c r="A687" t="inlineStr">
+    <row r="686">
+      <c r="A686" t="inlineStr">
         <is>
           <t xml:space="preserve">「初心者のためのスルス体書道トレーニング」
 تعليم خط الثلث للمبتدئين
@@ -14895,19 +14873,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B687" t="inlineStr">
+      <c r="B686" t="inlineStr">
         <is>
           <t>images/「初心者のためのスルス体書道トレーニン_img1.jpg</t>
         </is>
       </c>
-      <c r="C687" t="inlineStr">
+      <c r="C686" t="inlineStr">
         <is>
           <t>書道</t>
         </is>
       </c>
     </row>
-    <row r="688">
-      <c r="A688" t="inlineStr">
+    <row r="687">
+      <c r="A687" t="inlineStr">
         <is>
           <t xml:space="preserve">「笑顔でいなさい」خليك مبتسم
 カッリーク・ムブタスィム [Khallii-k mubtasim]
@@ -14916,19 +14894,19 @@
 2308 https://tmblr.co/Zj9tguYLXBvC </t>
         </is>
       </c>
-      <c r="B688" t="inlineStr">
+      <c r="B687" t="inlineStr">
         <is>
           <t>images/「笑顔でいなさい」_img1.jpg</t>
         </is>
       </c>
-      <c r="C688" t="inlineStr">
+      <c r="C687" t="inlineStr">
         <is>
           <t>スマイル ,名言</t>
         </is>
       </c>
     </row>
-    <row r="689">
-      <c r="A689" t="inlineStr">
+    <row r="688">
+      <c r="A688" t="inlineStr">
         <is>
           <t xml:space="preserve">自動車メーカー
 ⁦・「TOYOTA」( تويوتا )⁩
@@ -14940,19 +14918,19 @@
 2308 syarah com </t>
         </is>
       </c>
-      <c r="B689" t="inlineStr">
+      <c r="B688" t="inlineStr">
         <is>
           <t>images/自動車メーカー_img1.jpg,images/自動車メーカー_img2.jpg,images/自動車メーカー_img3.jpg,images/自動車メーカー_img4.jpg</t>
         </is>
       </c>
-      <c r="C689" t="inlineStr">
+      <c r="C688" t="inlineStr">
         <is>
           <t>日本車 ,韓国車</t>
         </is>
       </c>
     </row>
-    <row r="690">
-      <c r="A690" t="inlineStr">
+    <row r="689">
+      <c r="A689" t="inlineStr">
         <is>
           <t xml:space="preserve">「僕たちは協力して不可能を達成するよ」
 بالتعاون نحقق المحال
@@ -14962,19 +14940,19 @@
 2109 </t>
         </is>
       </c>
-      <c r="B690" t="inlineStr">
+      <c r="B689" t="inlineStr">
         <is>
           <t>images/「僕たちは協力して不可能を達成するよ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C690" t="inlineStr">
+      <c r="C689" t="inlineStr">
         <is>
           <t>無理 ,ハム太郎</t>
         </is>
       </c>
     </row>
-    <row r="691">
-      <c r="A691" t="inlineStr">
+    <row r="690">
+      <c r="A690" t="inlineStr">
         <is>
           <t xml:space="preserve">「幸せは伝染性。喜びを広めよう」
 السعادة معدية فأشع الفرح
@@ -14984,19 +14962,19 @@
 2511 instagram　com/p/fVEfxEo7Va/ </t>
         </is>
       </c>
-      <c r="B691" t="inlineStr">
+      <c r="B690" t="inlineStr">
         <is>
           <t>images/「幸せは伝染性。喜びを広めよう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C691" t="inlineStr">
+      <c r="C690" t="inlineStr">
         <is>
           <t>拡散希望</t>
         </is>
       </c>
     </row>
-    <row r="692">
-      <c r="A692" t="inlineStr">
+    <row r="691">
+      <c r="A691" t="inlineStr">
         <is>
           <t xml:space="preserve">「ストレスは人間だけのものではない」
 الشعور بالتوتر ليس حكرًا على البشر
@@ -15004,19 +14982,19 @@
 2408 https://x.com/NatGeoMagArab/status/1736755816911487420 </t>
         </is>
       </c>
-      <c r="B692" t="inlineStr">
+      <c r="B691" t="inlineStr">
         <is>
           <t>images/「ストレスは人間だけのものではない」_img1.jpg</t>
         </is>
       </c>
-      <c r="C692" t="inlineStr">
+      <c r="C691" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,ストレス</t>
         </is>
       </c>
     </row>
-    <row r="693">
-      <c r="A693" t="inlineStr">
+    <row r="692">
+      <c r="A692" t="inlineStr">
         <is>
           <t xml:space="preserve">「私達は出来ます！」
 نستطيع فعلها
@@ -15026,19 +15004,19 @@
 2308 NAHARBAHIJ com </t>
         </is>
       </c>
-      <c r="B693" t="inlineStr">
+      <c r="B692" t="inlineStr">
         <is>
           <t>images/「私達は出来ます！」_img1.jpg</t>
         </is>
       </c>
-      <c r="C693" t="inlineStr">
+      <c r="C692" t="inlineStr">
         <is>
           <t>女性 ,パロディ</t>
         </is>
       </c>
     </row>
-    <row r="694">
-      <c r="A694" t="inlineStr">
+    <row r="693">
+      <c r="A693" t="inlineStr">
         <is>
           <t xml:space="preserve">「全然分からん」ولا فاهم إشي
 ウラー・ファーヒム・イシ [w-laa faahim 'iShy]
@@ -15048,19 +15026,19 @@
 2209 出典不明 </t>
         </is>
       </c>
-      <c r="B694" t="inlineStr">
+      <c r="B693" t="inlineStr">
         <is>
           <t>images/「全然分からん」_img1.jpg</t>
         </is>
       </c>
-      <c r="C694" t="inlineStr">
+      <c r="C693" t="inlineStr">
         <is>
           <t>アラビア語</t>
         </is>
       </c>
     </row>
-    <row r="695">
-      <c r="A695" t="inlineStr">
+    <row r="694">
+      <c r="A694" t="inlineStr">
         <is>
           <t xml:space="preserve">「人間は一人ひとり、特別な才がある。だから自分を他人と比べるのはやめよう」
 لكل إنسان مواهبه الخاصة 
@@ -15069,19 +15047,19 @@
 1812 Gwid3 </t>
         </is>
       </c>
-      <c r="B695" t="inlineStr">
+      <c r="B694" t="inlineStr">
         <is>
           <t>images/「人間は一人ひとり、特別な才がある。だ_img1.jpg</t>
         </is>
       </c>
-      <c r="C695" t="inlineStr">
+      <c r="C694" t="inlineStr">
         <is>
           <t>自尊 ,プライド</t>
         </is>
       </c>
     </row>
-    <row r="696">
-      <c r="A696" t="inlineStr">
+    <row r="695">
+      <c r="A695" t="inlineStr">
         <is>
           <t xml:space="preserve">「デザイン」تَصْمِيمٌ
 タスミーム [ta_smiim(un)]
@@ -15089,19 +15067,19 @@
 1903 arabictypography com </t>
         </is>
       </c>
-      <c r="B696" t="inlineStr">
+      <c r="B695" t="inlineStr">
         <is>
           <t>images/「デザイン」_img1.jpg</t>
         </is>
       </c>
-      <c r="C696" t="inlineStr">
+      <c r="C695" t="inlineStr">
         <is>
           <t>文字 ,タイポグラフィー</t>
         </is>
       </c>
     </row>
-    <row r="697">
-      <c r="A697" t="inlineStr">
+    <row r="696">
+      <c r="A696" t="inlineStr">
         <is>
           <t xml:space="preserve">「この猫は食事をシェアするのが嫌い！」
 هذه القطة لا تحب مشاركة الطعام
@@ -15110,19 +15088,19 @@
 2605 facebook com/alahram/videos/2154923608133231/ </t>
         </is>
       </c>
-      <c r="B697" t="inlineStr">
+      <c r="B696" t="inlineStr">
         <is>
           <t>images/「この猫は食事をシェアするのが嫌い！」_img1.jpg</t>
         </is>
       </c>
-      <c r="C697" t="inlineStr">
+      <c r="C696" t="inlineStr">
         <is>
           <t>猫 ,ネコ</t>
         </is>
       </c>
     </row>
-    <row r="698">
-      <c r="A698" t="inlineStr">
+    <row r="697">
+      <c r="A697" t="inlineStr">
         <is>
           <t xml:space="preserve">「怪獣との戦いでは自分が怪獣化せぬよう警戒しなさい」
 احذر عند محاربة الوحوش ألا تصبح واحدا منهم
@@ -15132,19 +15110,19 @@
 2108 warag-3nb.tumblr </t>
         </is>
       </c>
-      <c r="B698" t="inlineStr">
+      <c r="B697" t="inlineStr">
         <is>
           <t>images/「怪獣との戦いでは自分が怪獣化せぬよう_img1.jpg,images/ 「怪獣との戦いでは自分が怪獣化せぬよう_img2.jpg</t>
         </is>
       </c>
-      <c r="C698" t="inlineStr">
+      <c r="C697" t="inlineStr">
         <is>
           <t>正気 ,モンスター</t>
         </is>
       </c>
     </row>
-    <row r="699">
-      <c r="A699" t="inlineStr">
+    <row r="698">
+      <c r="A698" t="inlineStr">
         <is>
           <t xml:space="preserve">「錯視アート」فن الخداع البصري
 ファンヌ_ルヒダーイ_ルバサリーイ [fannu l-Khidaa*i l-ba_sariyy]
@@ -15153,19 +15131,19 @@
 2409 https://online.pubhtml5.com/idtb/neft/ </t>
         </is>
       </c>
-      <c r="B699" t="inlineStr">
+      <c r="B698" t="inlineStr">
         <is>
           <t>images/「錯視アート」_img1.jpg</t>
         </is>
       </c>
-      <c r="C699" t="inlineStr">
+      <c r="C698" t="inlineStr">
         <is>
           <t>トリックアート</t>
         </is>
       </c>
     </row>
-    <row r="700">
-      <c r="A700" t="inlineStr">
+    <row r="699">
+      <c r="A699" t="inlineStr">
         <is>
           <t xml:space="preserve">「自然界の消防士の訓練」
 تدريبات رجال الإطفاء في الطبيعة
@@ -15173,19 +15151,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1462420543890608129 </t>
         </is>
       </c>
-      <c r="B700" t="inlineStr">
+      <c r="B699" t="inlineStr">
         <is>
           <t>images/「自然界の消防士の訓練」_img1.jpg,images/ 「自然界の消防士の訓練」_img2.jpg</t>
         </is>
       </c>
-      <c r="C700" t="inlineStr">
+      <c r="C699" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,ヒグマ</t>
         </is>
       </c>
     </row>
-    <row r="701">
-      <c r="A701" t="inlineStr">
+    <row r="700">
+      <c r="A700" t="inlineStr">
         <is>
           <t xml:space="preserve">「救助」إسعاف
 イスアーフ ['is*aaf]
@@ -15194,19 +15172,19 @@
 2109 ambulance gov ae </t>
         </is>
       </c>
-      <c r="B701" t="inlineStr">
+      <c r="B700" t="inlineStr">
         <is>
           <t>images/「救助」_img1.jpg</t>
         </is>
       </c>
-      <c r="C701" t="inlineStr">
+      <c r="C700" t="inlineStr">
         <is>
           <t>救急車 ,はたらくくるま</t>
         </is>
       </c>
     </row>
-    <row r="702">
-      <c r="A702" t="inlineStr">
+    <row r="701">
+      <c r="A701" t="inlineStr">
         <is>
           <t xml:space="preserve">「感情／感覚」الإحْسَاسْ
 アルイヒサース [al-'iHsaas]
@@ -15215,19 +15193,19 @@
 2308 iN49R </t>
         </is>
       </c>
-      <c r="B702" t="inlineStr">
+      <c r="B701" t="inlineStr">
         <is>
           <t>images/「感情／感覚」_img1.jpg</t>
         </is>
       </c>
-      <c r="C702" t="inlineStr">
+      <c r="C701" t="inlineStr">
         <is>
           <t>オフ ,一休み</t>
         </is>
       </c>
     </row>
-    <row r="703">
-      <c r="A703" t="inlineStr">
+    <row r="702">
+      <c r="A702" t="inlineStr">
         <is>
           <t xml:space="preserve">「ひらめき」إلهام
 イルハーム ['lhaam]
@@ -15239,19 +15217,19 @@
 2103 出典不明 </t>
         </is>
       </c>
-      <c r="B703" t="inlineStr">
+      <c r="B702" t="inlineStr">
         <is>
           <t>images/「ひらめき」_img1.jpg</t>
         </is>
       </c>
-      <c r="C703" t="inlineStr">
+      <c r="C702" t="inlineStr">
         <is>
           <t>アラビア語</t>
         </is>
       </c>
     </row>
-    <row r="704">
-      <c r="A704" t="inlineStr">
+    <row r="703">
+      <c r="A703" t="inlineStr">
         <is>
           <t xml:space="preserve">「Ibdaa／クリエイティビティ」
 إبداع
@@ -15260,19 +15238,19 @@
 2308 Ibdaa Design &amp; Decoration Office </t>
         </is>
       </c>
-      <c r="B704" t="inlineStr">
+      <c r="B703" t="inlineStr">
         <is>
           <t>images/「Ibdaa／クリエイティビティ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C704" t="inlineStr">
+      <c r="C703" t="inlineStr">
         <is>
           <t>創造性 ,独自性</t>
         </is>
       </c>
     </row>
-    <row r="705">
-      <c r="A705" t="inlineStr">
+    <row r="704">
+      <c r="A704" t="inlineStr">
         <is>
           <t xml:space="preserve">「奮闘なくして進歩なし」
 بدون كفاح لايوجد تقدم
@@ -15282,19 +15260,19 @@
 2105 ROUYMS TUMBLR COM </t>
         </is>
       </c>
-      <c r="B705" t="inlineStr">
+      <c r="B704" t="inlineStr">
         <is>
           <t>images/「奮闘なくして進歩なし」_img1.jpg</t>
         </is>
       </c>
-      <c r="C705" t="inlineStr">
+      <c r="C704" t="inlineStr">
         <is>
           <t>努力 ,三角形</t>
         </is>
       </c>
     </row>
-    <row r="706">
-      <c r="A706" t="inlineStr">
+    <row r="705">
+      <c r="A705" t="inlineStr">
         <is>
           <t xml:space="preserve">「木に登れば熊の危険を避けられるとお考えなら、考え直しましょう！」 
 إن اعتقدت أنك بمنأى عن خطر الدب عند تسلق الأشجار.. راجع حساباتك
@@ -15302,19 +15280,19 @@
 2202 NatGeoMagArab </t>
         </is>
       </c>
-      <c r="B706" t="inlineStr">
+      <c r="B705" t="inlineStr">
         <is>
           <t>images/「木に登れば熊の危険を避けられるとお考.jpeg</t>
         </is>
       </c>
-      <c r="C706" t="inlineStr">
+      <c r="C705" t="inlineStr">
         <is>
           <t>クマ</t>
         </is>
       </c>
     </row>
-    <row r="707">
-      <c r="A707" t="inlineStr">
+    <row r="706">
+      <c r="A706" t="inlineStr">
         <is>
           <t xml:space="preserve">「卒業おめでとう」مبروك التخرج
 マブルーク・タカッルジ [mabruuk a^taKharruj]
@@ -15323,19 +15301,19 @@
 2308 https://instagram.com/fatoomworld </t>
         </is>
       </c>
-      <c r="B707" t="inlineStr">
+      <c r="B706" t="inlineStr">
         <is>
           <t>images/「卒業おめでとう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C707" t="inlineStr">
+      <c r="C706" t="inlineStr">
         <is>
           <t>卒業 ,イラスト</t>
         </is>
       </c>
     </row>
-    <row r="708">
-      <c r="A708" t="inlineStr">
+    <row r="707">
+      <c r="A707" t="inlineStr">
         <is>
           <t xml:space="preserve">「停止距離の計算」
 حساب مسافة التوقف
@@ -15345,19 +15323,19 @@
 2109 assurance-auto-info </t>
         </is>
       </c>
-      <c r="B708" t="inlineStr">
+      <c r="B707" t="inlineStr">
         <is>
           <t>images/「停止距離の計算」_img1.jpg</t>
         </is>
       </c>
-      <c r="C708" t="inlineStr">
+      <c r="C707" t="inlineStr">
         <is>
           <t>保険 ,自動車</t>
         </is>
       </c>
     </row>
-    <row r="709">
-      <c r="A709" t="inlineStr">
+    <row r="708">
+      <c r="A708" t="inlineStr">
         <is>
           <t xml:space="preserve">「教師要らず：10日でフランス語会話」
 بدون معلم
@@ -15367,19 +15345,19 @@
 2308 englais-best com </t>
         </is>
       </c>
-      <c r="B709" t="inlineStr">
+      <c r="B708" t="inlineStr">
         <is>
           <t>images/「教師要らず：10日でフランス語会話」_img1.jpg</t>
         </is>
       </c>
-      <c r="C709" t="inlineStr">
+      <c r="C708" t="inlineStr">
         <is>
           <t>教師なし学習</t>
         </is>
       </c>
     </row>
-    <row r="710">
-      <c r="A710" t="inlineStr">
+    <row r="709">
+      <c r="A709" t="inlineStr">
         <is>
           <t xml:space="preserve">「衝突」تصادم
 タサードゥム [ta_saadum]
@@ -15388,19 +15366,19 @@
 1810 </t>
         </is>
       </c>
-      <c r="B710" t="inlineStr">
+      <c r="B709" t="inlineStr">
         <is>
           <t>images/「衝突」_img1.jpg</t>
         </is>
       </c>
-      <c r="C710" t="inlineStr">
+      <c r="C709" t="inlineStr">
         <is>
           <t>あらびあや</t>
         </is>
       </c>
     </row>
-    <row r="711">
-      <c r="A711" t="inlineStr">
+    <row r="710">
+      <c r="A710" t="inlineStr">
         <is>
           <t xml:space="preserve">「楽観主義」تَفَاؤُلٌ
 タファーウル [tafaa'ul(un)]
@@ -15409,19 +15387,19 @@
 1904 arabictypography com </t>
         </is>
       </c>
-      <c r="B711" t="inlineStr">
+      <c r="B710" t="inlineStr">
         <is>
           <t>images/「楽観主義」_img1.jpg</t>
         </is>
       </c>
-      <c r="C711" t="inlineStr">
+      <c r="C710" t="inlineStr">
         <is>
           <t>やわらか ,緑</t>
         </is>
       </c>
     </row>
-    <row r="712">
-      <c r="A712" t="inlineStr">
+    <row r="711">
+      <c r="A711" t="inlineStr">
         <is>
           <t xml:space="preserve">「シベリアジャコウジカは、絶滅の危機にあると見なされている」
 يعد "أيل المسك السيبيري" مهددًا بالانقراض
@@ -15429,19 +15407,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1320666649045790720 </t>
         </is>
       </c>
-      <c r="B712" t="inlineStr">
+      <c r="B711" t="inlineStr">
         <is>
           <t>images/「シベリアジャコウジカは、絶滅の危機に_img1.jpg,images/「シベリアジャコウジカは、絶滅の危機に_img2.jpg</t>
         </is>
       </c>
-      <c r="C712" t="inlineStr">
+      <c r="C711" t="inlineStr">
         <is>
           <t>手書き語学 ,シベリア</t>
         </is>
       </c>
     </row>
-    <row r="713">
-      <c r="A713" t="inlineStr">
+    <row r="712">
+      <c r="A712" t="inlineStr">
         <is>
           <t xml:space="preserve">「融合／折衷／フュージョン」
 انصهار
@@ -15450,38 +15428,38 @@
 1811 elmahdyart Instagram </t>
         </is>
       </c>
-      <c r="B713" t="inlineStr">
+      <c r="B712" t="inlineStr">
         <is>
           <t>images/「融合／折衷／フュージョン」_img1.jpg</t>
         </is>
       </c>
-      <c r="C713" t="inlineStr">
+      <c r="C712" t="inlineStr">
         <is>
           <t>カリグラフィー ,書道</t>
         </is>
       </c>
     </row>
-    <row r="714">
-      <c r="A714" t="inlineStr">
+    <row r="713">
+      <c r="A713" t="inlineStr">
         <is>
           <t xml:space="preserve">「この子供は、昼寝をしようとする母親を邪魔しているようだ」
 「場所はインドのトラ保護区、バンダウガル公園。トラは生態ピラミッドのトップの捕食動物だが、最もリスクの高い絶滅危惧種のひとつである」
 2308 https://twitter.com/natgeomagarab/status/1553681890665586689 </t>
         </is>
       </c>
-      <c r="B714" t="inlineStr">
+      <c r="B713" t="inlineStr">
         <is>
           <t>images/「この子供は、昼寝をしようとする母親を_img1.jpg,images/「この子供は、昼寝をしようとする母親を_img2.jpg</t>
         </is>
       </c>
-      <c r="C714" t="inlineStr">
+      <c r="C713" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,トラ</t>
         </is>
       </c>
     </row>
-    <row r="715">
-      <c r="A715" t="inlineStr">
+    <row r="714">
+      <c r="A714" t="inlineStr">
         <is>
           <t xml:space="preserve">「もし敬意が落ちたら、それと一緒に全部落ちるのだ」
 إن سقط الإحترام سقط معه كل شيء
@@ -15490,19 +15468,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B715" t="inlineStr">
+      <c r="B714" t="inlineStr">
         <is>
           <t>images/「もし敬意が落ちたら、それと一緒に全部_img1.jpg</t>
         </is>
       </c>
-      <c r="C715" t="inlineStr">
+      <c r="C714" t="inlineStr">
         <is>
           <t>リスペクト ,落書き</t>
         </is>
       </c>
     </row>
-    <row r="716">
-      <c r="A716" t="inlineStr">
+    <row r="715">
+      <c r="A715" t="inlineStr">
         <is>
           <t xml:space="preserve">「エジプト特許庁」
 مكتب براءات الاختراع المصرى
@@ -15512,19 +15490,19 @@
 2312 </t>
         </is>
       </c>
-      <c r="B716" t="inlineStr">
+      <c r="B715" t="inlineStr">
         <is>
           <t>images/「エジプト特許庁」_img1.jpg</t>
         </is>
       </c>
-      <c r="C716" t="inlineStr">
+      <c r="C715" t="inlineStr">
         <is>
           <t>patent</t>
         </is>
       </c>
     </row>
-    <row r="717">
-      <c r="A717" t="inlineStr">
+    <row r="716">
+      <c r="A716" t="inlineStr">
         <is>
           <t xml:space="preserve">「選挙」إنتخابات
 インティカーバート [intiKhaabaat]
@@ -15533,19 +15511,19 @@
 2311 nna-leb gov lb </t>
         </is>
       </c>
-      <c r="B717" t="inlineStr">
+      <c r="B716" t="inlineStr">
         <is>
           <t>images/「選挙」_img1.jpg</t>
         </is>
       </c>
-      <c r="C717" t="inlineStr">
+      <c r="C716" t="inlineStr">
         <is>
           <t>選挙 ,投票</t>
         </is>
       </c>
     </row>
-    <row r="718">
-      <c r="A718" t="inlineStr">
+    <row r="717">
+      <c r="A717" t="inlineStr">
         <is>
           <t xml:space="preserve">「待ちぼうけ」إنتظار
 インティザール [inti_Dhaar]
@@ -15554,19 +15532,19 @@
 1809 in4sser.tumblr </t>
         </is>
       </c>
-      <c r="B718" t="inlineStr">
+      <c r="B717" t="inlineStr">
         <is>
           <t>images/「待ちぼうけ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C718" t="inlineStr">
+      <c r="C717" t="inlineStr">
         <is>
           <t>遅すぎ ,辛抱</t>
         </is>
       </c>
     </row>
-    <row r="719">
-      <c r="A719" t="inlineStr">
+    <row r="718">
+      <c r="A718" t="inlineStr">
         <is>
           <t xml:space="preserve">「試験」إختبار
 イクティバール [iKhtibaar]
@@ -15575,19 +15553,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B719" t="inlineStr">
+      <c r="B718" t="inlineStr">
         <is>
           <t>images/「試験」_img1.jpg</t>
         </is>
       </c>
-      <c r="C719" t="inlineStr">
+      <c r="C718" t="inlineStr">
         <is>
           <t>テスト ,考査</t>
         </is>
       </c>
     </row>
-    <row r="720">
-      <c r="A720" t="inlineStr">
+    <row r="719">
+      <c r="A719" t="inlineStr">
         <is>
           <t xml:space="preserve">「チャンネル登録」اشتراك
 イシティラーク [iShtiraak]
@@ -15596,19 +15574,19 @@
 2308 </t>
         </is>
       </c>
-      <c r="B720" t="inlineStr">
+      <c r="B719" t="inlineStr">
         <is>
           <t>images/「チャンネル登録」_img1.jpg</t>
         </is>
       </c>
-      <c r="C720" t="inlineStr">
+      <c r="C719" t="inlineStr">
         <is>
           <t>Subscribe ,YouTube</t>
         </is>
       </c>
     </row>
-    <row r="721">
-      <c r="A721" t="inlineStr">
+    <row r="720">
+      <c r="A720" t="inlineStr">
         <is>
           <t xml:space="preserve">「スマイル」ابتسام
 イブティサーム [ibtisaam]
@@ -15616,37 +15594,37 @@
 1903 behance Written-Visuals </t>
         </is>
       </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>images/「スマイル」_img1.jpg</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>スマイリー ,ツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t xml:space="preserve">「身体の一部として…」
+2308 https://twitter.com/NatGeoMagArab/status/1528292080337813504 </t>
+        </is>
+      </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>images/「スマイル」_img1.jpg</t>
+          <t>images/「身体の一部として…」_img1.jpg</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>スマイリー ,ツ</t>
+          <t>手書き語学 ,カンガルー</t>
         </is>
       </c>
     </row>
     <row r="722">
       <c r="A722" t="inlineStr">
-        <is>
-          <t xml:space="preserve">「身体の一部として…」
-2308 https://twitter.com/NatGeoMagArab/status/1528292080337813504 </t>
-        </is>
-      </c>
-      <c r="B722" t="inlineStr">
-        <is>
-          <t>images/「身体の一部として…」_img1.jpg</t>
-        </is>
-      </c>
-      <c r="C722" t="inlineStr">
-        <is>
-          <t>手書き語学 ,カンガルー</t>
-        </is>
-      </c>
-    </row>
-    <row r="723">
-      <c r="A723" t="inlineStr">
         <is>
           <t xml:space="preserve">「ディスカバリー」إكتشاف
 イクティシャーフ [iktiShaaf]
@@ -15654,19 +15632,19 @@
 2308 tephanegabrielli com </t>
         </is>
       </c>
-      <c r="B723" t="inlineStr">
+      <c r="B722" t="inlineStr">
         <is>
           <t>images/「ディスカバリー」_img1.jpg</t>
         </is>
       </c>
-      <c r="C723" t="inlineStr">
+      <c r="C722" t="inlineStr">
         <is>
           <t>discovery ,デザイン</t>
         </is>
       </c>
     </row>
-    <row r="724">
-      <c r="A724" t="inlineStr">
+    <row r="723">
+      <c r="A723" t="inlineStr">
         <is>
           <t xml:space="preserve">「重力波の発見は新しい窓を開いた」
 فتَح اكتشاف موجات الجاذبية نافذة جديدة
@@ -15674,19 +15652,19 @@
 2308 https://twitter.com/SciTalk2U/status/1454891943440289793 </t>
         </is>
       </c>
-      <c r="B724" t="inlineStr">
+      <c r="B723" t="inlineStr">
         <is>
           <t>images/「重力波の発見は新しい窓を開いた」_img1.jpg</t>
         </is>
       </c>
-      <c r="C724" t="inlineStr">
+      <c r="C723" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,重力波</t>
         </is>
       </c>
     </row>
-    <row r="725">
-      <c r="A725" t="inlineStr">
+    <row r="724">
+      <c r="A724" t="inlineStr">
         <is>
           <t xml:space="preserve">「微笑みに微笑み。先にした人の方が美しい」
 الإبتسامة بالإبتسامة والبادئ أجمل
@@ -15695,19 +15673,19 @@
 2104 出典不明 </t>
         </is>
       </c>
-      <c r="B725" t="inlineStr">
+      <c r="B724" t="inlineStr">
         <is>
           <t>images/「微笑みに微笑み。先にした人の方が美し_img1.jpg,images/「微笑みに微笑み。先にした人の方が美し_img2.jpg</t>
         </is>
       </c>
-      <c r="C725" t="inlineStr">
+      <c r="C724" t="inlineStr">
         <is>
           <t>スマイル ,名言</t>
         </is>
       </c>
     </row>
-    <row r="726">
-      <c r="A726" t="inlineStr">
+    <row r="725">
+      <c r="A725" t="inlineStr">
         <is>
           <t xml:space="preserve">「笑顔」ابتسامة
 イブティサーマ [ibtisaama(tun)]
@@ -15716,19 +15694,19 @@
 2308 satokomatsu, minne </t>
         </is>
       </c>
-      <c r="B726" t="inlineStr">
+      <c r="B725" t="inlineStr">
         <is>
           <t>images/「笑顔」_img1.jpg</t>
         </is>
       </c>
-      <c r="C726" t="inlineStr">
+      <c r="C725" t="inlineStr">
         <is>
           <t>スマイル ,ツ</t>
         </is>
       </c>
     </row>
-    <row r="727">
-      <c r="A727" t="inlineStr">
+    <row r="726">
+      <c r="A726" t="inlineStr">
         <is>
           <t xml:space="preserve">「信仰」ايمان
 イーマーン ['iimaan]
@@ -15737,19 +15715,19 @@
 2506 instagram com/p/6ST-WHOOkJ/ </t>
         </is>
       </c>
-      <c r="B727" t="inlineStr">
+      <c r="B726" t="inlineStr">
         <is>
           <t>images/「信仰」_img1.jpg</t>
         </is>
       </c>
-      <c r="C727" t="inlineStr">
+      <c r="C726" t="inlineStr">
         <is>
           <t>宗教 ,信念</t>
         </is>
       </c>
     </row>
-    <row r="728">
-      <c r="A728" t="inlineStr">
+    <row r="727">
+      <c r="A727" t="inlineStr">
         <is>
           <t xml:space="preserve">「放送」إذاعة
 イザーア ['iDhaa*a]
@@ -15758,19 +15736,19 @@
 2404 heemades, Instagram </t>
         </is>
       </c>
-      <c r="B728" t="inlineStr">
+      <c r="B727" t="inlineStr">
         <is>
           <t>images/「放送」_img1.jpg</t>
         </is>
       </c>
-      <c r="C728" t="inlineStr">
+      <c r="C727" t="inlineStr">
         <is>
           <t>デザイン ,ラジオ</t>
         </is>
       </c>
     </row>
-    <row r="729">
-      <c r="A729" t="inlineStr">
+    <row r="728">
+      <c r="A728" t="inlineStr">
         <is>
           <t xml:space="preserve">「かきとりのちから」
 مهاراتي الإملائية
@@ -15779,19 +15757,19 @@
 2308 iqrawaoktoub.wordpress com </t>
         </is>
       </c>
-      <c r="B729" t="inlineStr">
+      <c r="B728" t="inlineStr">
         <is>
           <t>images/「かきとりのちから」_img1.jpg</t>
         </is>
       </c>
-      <c r="C729" t="inlineStr">
+      <c r="C728" t="inlineStr">
         <is>
           <t>国語 ,教材</t>
         </is>
       </c>
     </row>
-    <row r="730">
-      <c r="A730" t="inlineStr">
+    <row r="729">
+      <c r="A729" t="inlineStr">
         <is>
           <t xml:space="preserve">「歴史を作った男たち」
 رجال صنعوا التاريخ
@@ -15801,38 +15779,38 @@
 2410 https://x.gd/Wl5rJ </t>
         </is>
       </c>
-      <c r="B730" t="inlineStr">
+      <c r="B729" t="inlineStr">
         <is>
           <t>images/「歴史を作った男たち」_img1.jpg</t>
         </is>
       </c>
-      <c r="C730" t="inlineStr">
+      <c r="C729" t="inlineStr">
         <is>
           <t>偉人</t>
         </is>
       </c>
     </row>
-    <row r="731">
-      <c r="A731" t="inlineStr">
+    <row r="730">
+      <c r="A730" t="inlineStr">
         <is>
           <t xml:space="preserve">「無限の宇宙を旅した光」
 「何百年もの末にジェイムズ・ウェッブ望遠鏡のレンズの上に落ち、我々に遠い宇宙の美しさを見せてくれる。最も純粋な形と最も素晴らしい姿で」
 2308 https://twitter.com/NatGeoMagArab/status/1557811592636485632 </t>
         </is>
       </c>
-      <c r="B731" t="inlineStr">
+      <c r="B730" t="inlineStr">
         <is>
           <t>images/「無限の宇宙を旅した光」_img1.jpg</t>
         </is>
       </c>
-      <c r="C731" t="inlineStr">
+      <c r="C730" t="inlineStr">
         <is>
           <t>手書き語学 ,宇宙</t>
         </is>
       </c>
     </row>
-    <row r="732">
-      <c r="A732" t="inlineStr">
+    <row r="731">
+      <c r="A731" t="inlineStr">
         <is>
           <t xml:space="preserve">「日本好きになり行きたくなる20項」
 عشرون شيئا يجعلك تحب اليابان وترغب في زيارتها
@@ -15841,19 +15819,19 @@
 2308 wattpad </t>
         </is>
       </c>
-      <c r="B732" t="inlineStr">
+      <c r="B731" t="inlineStr">
         <is>
           <t>images/「日本好きになり行きたくなる20項」_img1.jpg</t>
         </is>
       </c>
-      <c r="C732" t="inlineStr">
+      <c r="C731" t="inlineStr">
         <is>
           <t>اليابان ,Japan</t>
         </is>
       </c>
     </row>
-    <row r="733">
-      <c r="A733" t="inlineStr">
+    <row r="732">
+      <c r="A732" t="inlineStr">
         <is>
           <t xml:space="preserve">「ピッタリの瞬間に撮影され、ドラゴンが火を噴いているように見える」
 التُقطت في اللحظة المناسبة لتبدو مثل تنين ينفث اللهب
@@ -15861,19 +15839,19 @@
 2509 https://twitter.com/NatGeoMagArab/status/1588780660269150208 </t>
         </is>
       </c>
-      <c r="B733" t="inlineStr">
+      <c r="B732" t="inlineStr">
         <is>
           <t>images/「ピッタリの瞬間に撮影され、ドラゴンが_img1.jpg,images/ 「ピッタリの瞬間に撮影され、ドラゴンが_img2.jpg</t>
         </is>
       </c>
-      <c r="C733" t="inlineStr">
+      <c r="C732" t="inlineStr">
         <is>
           <t xml:space="preserve">ドラゴン </t>
         </is>
       </c>
     </row>
-    <row r="734">
-      <c r="A734" t="inlineStr">
+    <row r="733">
+      <c r="A733" t="inlineStr">
         <is>
           <t xml:space="preserve">「満足は不滅の宝である」
 القَناعَةُ كنز لا يَفنَى
@@ -15883,55 +15861,55 @@
 2308 kareem mrghani </t>
         </is>
       </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>images/「満足は不滅の宝である」_img1.jpg</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>幸福度</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ゴシキセイガイインコ。
+2409 https://twitter.com/NatGeoMagArab/status/1600022262014676992 </t>
+        </is>
+      </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>images/「満足は不滅の宝である」_img1.jpg</t>
+          <t>images/ゴシキセイガイインコ。_img1.jpg</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>幸福度</t>
+          <t>手書き語学 ,アラビア語,オウム</t>
         </is>
       </c>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr">
         <is>
-          <t xml:space="preserve">ゴシキセイガイインコ。
-2409 https://twitter.com/NatGeoMagArab/status/1600022262014676992 </t>
+          <t xml:space="preserve">モモンガ。
+2403 https://twitter.com/NatGeoMagArab/status/1552541872966344704 </t>
         </is>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>images/ゴシキセイガイインコ。_img1.jpg</t>
+          <t>images/モモンガ。_img1.jpg,images/ モモンガ。_img2.jpg</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>手書き語学 ,アラビア語,オウム</t>
+          <t>手書き語学 ,アラビア語 ,モモンガ</t>
         </is>
       </c>
     </row>
     <row r="736">
       <c r="A736" t="inlineStr">
-        <is>
-          <t xml:space="preserve">モモンガ。
-2403 https://twitter.com/NatGeoMagArab/status/1552541872966344704 </t>
-        </is>
-      </c>
-      <c r="B736" t="inlineStr">
-        <is>
-          <t>images/モモンガ。_img1.jpg,images/ モモンガ。_img2.jpg</t>
-        </is>
-      </c>
-      <c r="C736" t="inlineStr">
-        <is>
-          <t>手書き語学 ,アラビア語 ,モモンガ</t>
-        </is>
-      </c>
-    </row>
-    <row r="737">
-      <c r="A737" t="inlineStr">
         <is>
           <t xml:space="preserve">「象の群れ。ドローンの音から逃げている」
 قطيع من الفيلة يفر هاربًا من صوت الدرون
@@ -15943,56 +15921,56 @@
 2009 https://twitter.com/NatGeoMagArab/status/1302970033627258881 </t>
         </is>
       </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>images/「象の群れ。ドローンの音から逃げている.jpg</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>ゾウ ,ドローン</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t xml:space="preserve">カルマン線。
+2308 https://twitter.com/NatGeoMagArab/status/1536436999522881536 </t>
+        </is>
+      </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>images/「象の群れ。ドローンの音から逃げている.jpg</t>
+          <t>images/カルマン線。_img1.jpg</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>ゾウ ,ドローン</t>
+          <t xml:space="preserve">手書き語学 ,アラビア語 ,宇宙 </t>
         </is>
       </c>
     </row>
     <row r="738">
       <c r="A738" t="inlineStr">
-        <is>
-          <t xml:space="preserve">カルマン線。
-2308 https://twitter.com/NatGeoMagArab/status/1536436999522881536 </t>
-        </is>
-      </c>
-      <c r="B738" t="inlineStr">
-        <is>
-          <t>images/カルマン線。_img1.jpg</t>
-        </is>
-      </c>
-      <c r="C738" t="inlineStr">
-        <is>
-          <t xml:space="preserve">手書き語学 ,アラビア語 ,宇宙 </t>
-        </is>
-      </c>
-    </row>
-    <row r="739">
-      <c r="A739" t="inlineStr">
         <is>
           <t xml:space="preserve">「恥ずかしがり屋のマヌルネコと暖かい朝の太陽光線」
 ⁦「二つの美しいもの」[Shay'-ayni jamiil-ayni] 属格：「物」( شيء )[Shay']・「美しい」( جميل )[jamiil]⁩
 2309 https://twitter.com/NatGeoMagArab/status/1697512148820504912 </t>
         </is>
       </c>
-      <c r="B739" t="inlineStr">
+      <c r="B738" t="inlineStr">
         <is>
           <t>images/「恥ずかしがり屋のマヌルネコと暖かい朝_img1.jpg</t>
         </is>
       </c>
-      <c r="C739" t="inlineStr">
+      <c r="C738" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,マヌルネコ</t>
         </is>
       </c>
     </row>
-    <row r="740">
-      <c r="A740" t="inlineStr">
+    <row r="739">
+      <c r="A739" t="inlineStr">
         <is>
           <t xml:space="preserve">「二回失敗しているペンギン」
 بطريق يفشل مرتين
@@ -16002,19 +15980,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1479483133766426626 </t>
         </is>
       </c>
-      <c r="B740" t="inlineStr">
+      <c r="B739" t="inlineStr">
         <is>
           <t>images/「二回失敗しているペンギン」_img1.jpg</t>
         </is>
       </c>
-      <c r="C740" t="inlineStr">
+      <c r="C739" t="inlineStr">
         <is>
           <t>ペンギン ,動物</t>
         </is>
       </c>
     </row>
-    <row r="741">
-      <c r="A741" t="inlineStr">
+    <row r="740">
+      <c r="A740" t="inlineStr">
         <is>
           <t xml:space="preserve">「2億光年の彼方できらめく炎と光」
 وهج ووميض يتلألأ على بعد 200 مليون سنة ضوئية
@@ -16025,15 +16003,15 @@
 2010 https://twitter.com/NatGeoMagArab/status/1303415502673342464 </t>
         </is>
       </c>
-      <c r="B741" t="inlineStr"/>
-      <c r="C741" t="inlineStr">
+      <c r="B740" t="inlineStr"/>
+      <c r="C740" t="inlineStr">
         <is>
           <t>宇宙 ,銀河</t>
         </is>
       </c>
     </row>
-    <row r="742">
-      <c r="A742" t="inlineStr">
+    <row r="741">
+      <c r="A741" t="inlineStr">
         <is>
           <t xml:space="preserve">「さまよう黒猫」قطة سوداء تجوب
 キッタトゥン・サウダーウ・タジューブ [qi^_tatun sawdaa'u ta-juub]
@@ -16042,19 +16020,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1532973177453760512 </t>
         </is>
       </c>
-      <c r="B742" t="inlineStr">
+      <c r="B741" t="inlineStr">
         <is>
           <t>images/「さまよう黒猫」_img1.jpg,images/ 「さまよう黒猫」_img2.jpg</t>
         </is>
       </c>
-      <c r="C742" t="inlineStr">
+      <c r="C741" t="inlineStr">
         <is>
           <t xml:space="preserve">手書き語学 ,モロッコ </t>
         </is>
       </c>
     </row>
-    <row r="743">
-      <c r="A743" t="inlineStr">
+    <row r="742">
+      <c r="A742" t="inlineStr">
         <is>
           <t xml:space="preserve">「サイのざらざらした皮を利用して自分の体を掻くネコ」
 قطة تستغل جلد الكركدن الخشن لحك جسدها
@@ -16063,19 +16041,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1476855740929216517 </t>
         </is>
       </c>
-      <c r="B743" t="inlineStr">
+      <c r="B742" t="inlineStr">
         <is>
           <t>images/「サイのざらざらした皮を利用して自分の_img1.jpg</t>
         </is>
       </c>
-      <c r="C743" t="inlineStr">
+      <c r="C742" t="inlineStr">
         <is>
           <t>サイ ,チェコ</t>
         </is>
       </c>
     </row>
-    <row r="744">
-      <c r="A744" t="inlineStr">
+    <row r="743">
+      <c r="A743" t="inlineStr">
         <is>
           <t xml:space="preserve">「沈まぬ太陽」شمس لا تغيب
 シャムス・ラー・タギーブ [Shams laa ta-Ghiib]
@@ -16084,19 +16062,19 @@
 2308 AHMED ELASSAL </t>
         </is>
       </c>
-      <c r="B744" t="inlineStr">
+      <c r="B743" t="inlineStr">
         <is>
           <t>images/「沈まぬ太陽」_img1.jpg</t>
         </is>
       </c>
-      <c r="C744" t="inlineStr">
+      <c r="C743" t="inlineStr">
         <is>
           <t>帝国 ,白夜</t>
         </is>
       </c>
     </row>
-    <row r="745">
-      <c r="A745" t="inlineStr">
+    <row r="744">
+      <c r="A744" t="inlineStr">
         <is>
           <t xml:space="preserve">「子供に食べさせている忍耐強い母親」
 أم صبورة تطعم صغيرها
@@ -16105,19 +16083,19 @@
 2308 https://twitter.com/natgeomagarab/status/1585572054509957120 </t>
         </is>
       </c>
-      <c r="B745" t="inlineStr">
+      <c r="B744" t="inlineStr">
         <is>
           <t>images/「子供に食べさせている忍耐強い母親」_img1.jpg</t>
         </is>
       </c>
-      <c r="C745" t="inlineStr">
+      <c r="C744" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,ミヤコドリ</t>
         </is>
       </c>
     </row>
-    <row r="746">
-      <c r="A746" t="inlineStr">
+    <row r="745">
+      <c r="A745" t="inlineStr">
         <is>
           <t xml:space="preserve">「コーヒーは繰り返さない恋物語」
 القهوة قصة عشق لن تتكرر
@@ -16127,19 +16105,19 @@
 2403 pin it/7tvd8Wc </t>
         </is>
       </c>
-      <c r="B746" t="inlineStr">
+      <c r="B745" t="inlineStr">
         <is>
           <t>images/「コーヒーは繰り返さない恋物語」_img1.jpg</t>
         </is>
       </c>
-      <c r="C746" t="inlineStr">
+      <c r="C745" t="inlineStr">
         <is>
           <t>コーヒー ,名言</t>
         </is>
       </c>
     </row>
-    <row r="747">
-      <c r="A747" t="inlineStr">
+    <row r="746">
+      <c r="A746" t="inlineStr">
         <is>
           <t xml:space="preserve">「星々で飾られた空。魅惑的な色合いで黄昏の美を満たしている」
 سماء مرصعة بالنجوم تضفي لمسة سحرية على جمال الشفق
@@ -16147,19 +16125,19 @@
 2010 https://twitter.com/NatGeoMagArab/status/1303777701975584768 </t>
         </is>
       </c>
-      <c r="B747" t="inlineStr">
+      <c r="B746" t="inlineStr">
         <is>
           <t>images/「星々で飾られた空。魅惑的な色合いで黄.png</t>
         </is>
       </c>
-      <c r="C747" t="inlineStr">
+      <c r="C746" t="inlineStr">
         <is>
           <t>星空 ,宇宙</t>
         </is>
       </c>
     </row>
-    <row r="748">
-      <c r="A748" t="inlineStr">
+    <row r="747">
+      <c r="A747" t="inlineStr">
         <is>
           <t xml:space="preserve">「国際宇宙ステーションからの写真。巨大な台風『ハイシェン（海神）』を映している」
 لقطات من محطة الفضاء الدولية تظهر إعصار "هايشن" الهائل
@@ -16167,19 +16145,19 @@
 2403 https://twitter.com/NatGeoMagArab/status/1302871968522235904 </t>
         </is>
       </c>
-      <c r="B748" t="inlineStr">
+      <c r="B747" t="inlineStr">
         <is>
           <t>images/「国際宇宙ステーションからの写真。巨大.png</t>
         </is>
       </c>
-      <c r="C748" t="inlineStr">
+      <c r="C747" t="inlineStr">
         <is>
           <t>台風</t>
         </is>
       </c>
     </row>
-    <row r="749">
-      <c r="A749" t="inlineStr">
+    <row r="748">
+      <c r="A748" t="inlineStr">
         <is>
           <t xml:space="preserve">「草を食む幸運な子羊たち」
 خراف محظوظة ترعى
@@ -16189,19 +16167,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1490211393554972676 </t>
         </is>
       </c>
-      <c r="B749" t="inlineStr">
+      <c r="B748" t="inlineStr">
         <is>
           <t>images/「草を食む幸運な子羊たち」_img1.jpg,images/ 「草を食む幸運な子羊たち」_img2.jpg</t>
         </is>
       </c>
-      <c r="C749" t="inlineStr">
+      <c r="C748" t="inlineStr">
         <is>
           <t>羊 ,アイルランド</t>
         </is>
       </c>
     </row>
-    <row r="750">
-      <c r="A750" t="inlineStr">
+    <row r="749">
+      <c r="A749" t="inlineStr">
         <is>
           <t xml:space="preserve">「お金で買えぬ10のもの」
 ١٠ أشياء لا تشترى بالمال
@@ -16211,19 +16189,19 @@
 2308 ayb124 </t>
         </is>
       </c>
-      <c r="B750" t="inlineStr">
+      <c r="B749" t="inlineStr">
         <is>
           <t>images/「お金で買えぬ10のもの」_img1.jpg</t>
         </is>
       </c>
-      <c r="C750" t="inlineStr">
+      <c r="C749" t="inlineStr">
         <is>
           <t>価値 ,購買</t>
         </is>
       </c>
     </row>
-    <row r="751">
-      <c r="A751" t="inlineStr">
+    <row r="750">
+      <c r="A750" t="inlineStr">
         <is>
           <t xml:space="preserve">「お金では買えないよ」
 هي أشْيَاءٌ لا تُشْتَرَى
@@ -16233,19 +16211,19 @@
 1906 mardy_zaawely, Instagram </t>
         </is>
       </c>
-      <c r="B751" t="inlineStr">
+      <c r="B750" t="inlineStr">
         <is>
           <t>images/「お金では買えないよ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C751" t="inlineStr">
+      <c r="C750" t="inlineStr">
         <is>
           <t>マスターカード ,価値</t>
         </is>
       </c>
     </row>
-    <row r="752">
-      <c r="A752" t="inlineStr">
+    <row r="751">
+      <c r="A751" t="inlineStr">
         <is>
           <t xml:space="preserve">「好奇心旺盛なホッキョクギツネ」
 ثعلب قطبي يملؤه الفضول
@@ -16255,15 +16233,15 @@
 2308 https://twitter.com/natgeomagarab/status/1157592172968808449 </t>
         </is>
       </c>
-      <c r="B752" t="inlineStr"/>
-      <c r="C752" t="inlineStr">
+      <c r="B751" t="inlineStr"/>
+      <c r="C751" t="inlineStr">
         <is>
           <t>ファーストコンタクト ,キツネ</t>
         </is>
       </c>
     </row>
-    <row r="753">
-      <c r="A753" t="inlineStr">
+    <row r="752">
+      <c r="A752" t="inlineStr">
         <is>
           <t xml:space="preserve">「グレンダイザーのいる国は死にません」
 لنْ يَموتَ شَعبٌ لدَيهِ غرندايزر
@@ -16272,56 +16250,56 @@
 2308 https://www.aljarida.com/articles/1462241741574732100/ </t>
         </is>
       </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>images/「グレンダイザーのいる国は死にません」_img1.jpg</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>UFOロボ ,アニメ</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t xml:space="preserve">「凍結路面を運転中、彼女は嫌な場面に居合わせた」
+2408 https://twitter.com/NatGeoMagArab/status/1610305209657626625 </t>
+        </is>
+      </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>images/「グレンダイザーのいる国は死にません」_img1.jpg</t>
+          <t>images/「凍結路面を運転中、彼女は嫌な場面に居_img1.jpg</t>
         </is>
       </c>
       <c r="C753" t="inlineStr">
         <is>
-          <t>UFOロボ ,アニメ</t>
+          <t>手書き語学 ,アラビア語 ,路面凍結</t>
         </is>
       </c>
     </row>
     <row r="754">
       <c r="A754" t="inlineStr">
-        <is>
-          <t xml:space="preserve">「凍結路面を運転中、彼女は嫌な場面に居合わせた」
-2408 https://twitter.com/NatGeoMagArab/status/1610305209657626625 </t>
-        </is>
-      </c>
-      <c r="B754" t="inlineStr">
-        <is>
-          <t>images/「凍結路面を運転中、彼女は嫌な場面に居_img1.jpg</t>
-        </is>
-      </c>
-      <c r="C754" t="inlineStr">
-        <is>
-          <t>手書き語学 ,アラビア語 ,路面凍結</t>
-        </is>
-      </c>
-    </row>
-    <row r="755">
-      <c r="A755" t="inlineStr">
         <is>
           <t xml:space="preserve">「虹が美しさを加えている、アルパカという動物の美しいショット」
 ⁦「美しいショット」[laq_tatun jamiilatun]：「ショット」( لقطة )[laq_ta]：( ـلٌ )[-lun]・( ـقٌ )[-qun]・( ـطٌ )[-_tun]・( ـةٌ )[-tun]⁩
 2308 https://twitter.com/natgeomagarab/status/1155115655928004608 </t>
         </is>
       </c>
-      <c r="B755" t="inlineStr">
+      <c r="B754" t="inlineStr">
         <is>
           <t>images/「虹が美しさを加えている、アルパカとい_img1.jpg</t>
         </is>
       </c>
-      <c r="C755" t="inlineStr">
+      <c r="C754" t="inlineStr">
         <is>
           <t>モフモフ ,アルパカ</t>
         </is>
       </c>
     </row>
-    <row r="756">
-      <c r="A756" t="inlineStr">
+    <row r="755">
+      <c r="A755" t="inlineStr">
         <is>
           <t xml:space="preserve">「幸せは…全然思いもよらない所からやって来る」
 السعادة تأتينا من أماكن لم نكن نتوقعها أبداً
@@ -16330,19 +16308,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B756" t="inlineStr">
+      <c r="B755" t="inlineStr">
         <is>
           <t>images/「幸せは…全然思いもよらない所からやっ_img1.jpg,images/ 「幸せは…全然思いもよらない所からやっ_img2.jpg</t>
         </is>
       </c>
-      <c r="C756" t="inlineStr">
+      <c r="C755" t="inlineStr">
         <is>
           <t>訪れ ,予想</t>
         </is>
       </c>
     </row>
-    <row r="757">
-      <c r="A757" t="inlineStr">
+    <row r="756">
+      <c r="A756" t="inlineStr">
         <is>
           <t xml:space="preserve">「あらゆる問題は、食べ物が解決してくれる」
 كل مشكلة ولها أكلة تحلها
@@ -16351,19 +16329,19 @@
 1909 ALQA AN 878 </t>
         </is>
       </c>
-      <c r="B757" t="inlineStr">
+      <c r="B756" t="inlineStr">
         <is>
           <t>images/「あらゆる問題は、食べ物が解決してくれ_img1.jpg</t>
         </is>
       </c>
-      <c r="C757" t="inlineStr">
+      <c r="C756" t="inlineStr">
         <is>
           <t>ストレス ,精神</t>
         </is>
       </c>
     </row>
-    <row r="758">
-      <c r="A758" t="inlineStr">
+    <row r="757">
+      <c r="A757" t="inlineStr">
         <is>
           <t xml:space="preserve">「冬で私が好きな物」
 أشياء أحبها بالشتاء
@@ -16373,19 +16351,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B758" t="inlineStr">
+      <c r="B757" t="inlineStr">
         <is>
           <t>images/「冬で私が好きな物」_img1.jpg</t>
         </is>
       </c>
-      <c r="C758" t="inlineStr">
+      <c r="C757" t="inlineStr">
         <is>
           <t>季節 ,冬</t>
         </is>
       </c>
     </row>
-    <row r="759">
-      <c r="A759" t="inlineStr">
+    <row r="758">
+      <c r="A758" t="inlineStr">
         <is>
           <t xml:space="preserve">「お金で買うことの出来ない物」
 أشياء لا تستطيع شراءها بالمال
@@ -16395,19 +16373,19 @@
 2409 https://x.com/akhbarak/status/1038402708414373888 </t>
         </is>
       </c>
-      <c r="B759" t="inlineStr">
+      <c r="B758" t="inlineStr">
         <is>
           <t>images/「お金で買うことの出来ない物」_img1.jpg,images/ 「お金で買うことの出来ない物」_img2.jpg</t>
         </is>
       </c>
-      <c r="C759" t="inlineStr">
+      <c r="C758" t="inlineStr">
         <is>
           <t>ショッピング ,価値</t>
         </is>
       </c>
     </row>
-    <row r="760">
-      <c r="A760" t="inlineStr">
+    <row r="759">
+      <c r="A759" t="inlineStr">
         <is>
           <t xml:space="preserve">「私たちが愛する言葉」
 كلماتٌ نُحبّها
@@ -16417,19 +16395,19 @@
 2109 جليل خزعل </t>
         </is>
       </c>
-      <c r="B760" t="inlineStr">
+      <c r="B759" t="inlineStr">
         <is>
           <t>images/「私たちが愛する言葉」_img1.jpg</t>
         </is>
       </c>
-      <c r="C760" t="inlineStr">
+      <c r="C759" t="inlineStr">
         <is>
           <t>花 ,贈り物</t>
         </is>
       </c>
     </row>
-    <row r="761">
-      <c r="A761" t="inlineStr">
+    <row r="760">
+      <c r="A760" t="inlineStr">
         <is>
           <t xml:space="preserve">「お茶についてあなたが知らない10の事実」
 عشر معلومات لا تعرفها عن الشاي
@@ -16438,19 +16416,19 @@
 2012 http://ara.tv/6syq2 </t>
         </is>
       </c>
-      <c r="B761" t="inlineStr">
+      <c r="B760" t="inlineStr">
         <is>
           <t>images/「お茶についてあなたが知らない10の事_img1.jpg</t>
         </is>
       </c>
-      <c r="C761" t="inlineStr">
+      <c r="C760" t="inlineStr">
         <is>
           <t>神農</t>
         </is>
       </c>
     </row>
-    <row r="762">
-      <c r="A762" t="inlineStr">
+    <row r="761">
+      <c r="A761" t="inlineStr">
         <is>
           <t xml:space="preserve">「大きくなったウソ」
 الكذبة الّتي كبرت
@@ -16460,19 +16438,19 @@
 2509 سلسلة الحلزونة </t>
         </is>
       </c>
-      <c r="B762" t="inlineStr">
+      <c r="B761" t="inlineStr">
         <is>
           <t>images/「大きくなったウソ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C762" t="inlineStr">
+      <c r="C761" t="inlineStr">
         <is>
           <t>絵本</t>
         </is>
       </c>
     </row>
-    <row r="763">
-      <c r="A763" t="inlineStr">
+    <row r="762">
+      <c r="A762" t="inlineStr">
         <is>
           <t xml:space="preserve">「自分に合った掃除機を買うには？」
 كيف تشتري المكنسة الكهربائية التي تناسبك؟
@@ -16481,19 +16459,19 @@
 2106 ts3a com </t>
         </is>
       </c>
-      <c r="B763" t="inlineStr">
+      <c r="B762" t="inlineStr">
         <is>
           <t>images/「自分に合った掃除機を買うには？」_img1.jpg</t>
         </is>
       </c>
-      <c r="C763" t="inlineStr">
+      <c r="C762" t="inlineStr">
         <is>
           <t>家電 ,掃除</t>
         </is>
       </c>
     </row>
-    <row r="764">
-      <c r="A764" t="inlineStr">
+    <row r="763">
+      <c r="A763" t="inlineStr">
         <is>
           <t xml:space="preserve">「仮にこれが批判の数としよう」
 لنفرض ان عدد الذين ينتقدونك
@@ -16504,19 +16482,19 @@
 2504 出典不明 </t>
         </is>
       </c>
-      <c r="B764" t="inlineStr">
+      <c r="B763" t="inlineStr">
         <is>
           <t>images/「仮にこれが批判の数としよう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C764" t="inlineStr">
+      <c r="C763" t="inlineStr">
         <is>
           <t>アンチ</t>
         </is>
       </c>
     </row>
-    <row r="765">
-      <c r="A765" t="inlineStr">
+    <row r="764">
+      <c r="A764" t="inlineStr">
         <is>
           <t xml:space="preserve">「ここに見えるのは何？」
 ما الذي تراه هنا؟
@@ -16526,15 +16504,15 @@
 2204 https://twitter.com/NatGeoMagArab/status/1506933850617700352 </t>
         </is>
       </c>
-      <c r="B765" t="inlineStr"/>
-      <c r="C765" t="inlineStr">
+      <c r="B764" t="inlineStr"/>
+      <c r="C764" t="inlineStr">
         <is>
           <t xml:space="preserve">ペンギン </t>
         </is>
       </c>
     </row>
-    <row r="766">
-      <c r="A766" t="inlineStr">
+    <row r="765">
+      <c r="A765" t="inlineStr">
         <is>
           <t xml:space="preserve">「今日辛いこと、明日は平気だろう」
 ما يؤلم اليوم سيهون غدًا
@@ -16544,19 +16522,19 @@
 2308 basmahjeff </t>
         </is>
       </c>
-      <c r="B766" t="inlineStr">
+      <c r="B765" t="inlineStr">
         <is>
           <t>images/「今日辛いこと、明日は平気だろう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C766" t="inlineStr">
+      <c r="C765" t="inlineStr">
         <is>
           <t>悩み ,達観</t>
         </is>
       </c>
     </row>
-    <row r="767">
-      <c r="A767" t="inlineStr">
+    <row r="766">
+      <c r="A766" t="inlineStr">
         <is>
           <t xml:space="preserve">「自分のすることを好きでなきゃ」
 عليك أن تحب ما تفعل
@@ -16565,19 +16543,19 @@
 1810 Ahmed Elhakeem </t>
         </is>
       </c>
-      <c r="B767" t="inlineStr">
+      <c r="B766" t="inlineStr">
         <is>
           <t>images/「自分のすることを好きでなきゃ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C767" t="inlineStr">
+      <c r="C766" t="inlineStr">
         <is>
           <t>転職 ,かわいい</t>
         </is>
       </c>
     </row>
-    <row r="768">
-      <c r="A768" t="inlineStr">
+    <row r="767">
+      <c r="A767" t="inlineStr">
         <is>
           <t xml:space="preserve">「この地上に生き甲斐あり」
 على هذه الأرض ما يستحق الحياة
@@ -16587,19 +16565,19 @@
 2308 Mahmoud Gafar </t>
         </is>
       </c>
-      <c r="B768" t="inlineStr">
+      <c r="B767" t="inlineStr">
         <is>
           <t>images/「この地上に生き甲斐あり」_img1.jpg</t>
         </is>
       </c>
-      <c r="C768" t="inlineStr">
+      <c r="C767" t="inlineStr">
         <is>
           <t>詩</t>
         </is>
       </c>
     </row>
-    <row r="769">
-      <c r="A769" t="inlineStr">
+    <row r="768">
+      <c r="A768" t="inlineStr">
         <is>
           <t xml:space="preserve">「おそらく、あなたの求めるものはあるだろう」
 لعلَّ ما تَرجوهُ سيَكونُ
@@ -16609,19 +16587,19 @@
 2308 PIXEL Instagram </t>
         </is>
       </c>
-      <c r="B769" t="inlineStr">
+      <c r="B768" t="inlineStr">
         <is>
           <t>images/「おそらく、あなたの求めるものはあるだ_img1.jpg</t>
         </is>
       </c>
-      <c r="C769" t="inlineStr">
+      <c r="C768" t="inlineStr">
         <is>
           <t>願い ,信仰</t>
         </is>
       </c>
     </row>
-    <row r="770">
-      <c r="A770" t="inlineStr">
+    <row r="769">
+      <c r="A769" t="inlineStr">
         <is>
           <t xml:space="preserve">「オレンジの効能が何か知っていますか？」
 هل تعرف ما هي فوائد البرتقال؟
@@ -16631,19 +16609,19 @@
 2308 sadahadhramowt com </t>
         </is>
       </c>
-      <c r="B770" t="inlineStr">
+      <c r="B769" t="inlineStr">
         <is>
           <t>images/「オレンジの効能が何か知っていますか？_img1.jpg</t>
         </is>
       </c>
-      <c r="C770" t="inlineStr">
+      <c r="C769" t="inlineStr">
         <is>
           <t>オレンジ ,フルーツ</t>
         </is>
       </c>
     </row>
-    <row r="771">
-      <c r="A771" t="inlineStr">
+    <row r="770">
+      <c r="A770" t="inlineStr">
         <is>
           <t xml:space="preserve">「遊ぶパンダの光景より可愛いものがありますか？」
 هل هناك ما هو ألطف من مشاهدة الباندا وهي تلعب؟
@@ -16651,19 +16629,19 @@
 2308 https://twitter.com/NatGeoMagArab/status/1494612797858074626 </t>
         </is>
       </c>
-      <c r="B771" t="inlineStr">
+      <c r="B770" t="inlineStr">
         <is>
           <t>images/「遊ぶパンダの光景より可愛いものがあり_img1.jpg</t>
         </is>
       </c>
-      <c r="C771" t="inlineStr">
+      <c r="C770" t="inlineStr">
         <is>
           <t>パンダ ,モコモコ</t>
         </is>
       </c>
     </row>
-    <row r="772">
-      <c r="A772" t="inlineStr">
+    <row r="771">
+      <c r="A771" t="inlineStr">
         <is>
           <t xml:space="preserve">「大事なのは何者だったかじゃない。何者になるかだ」
 ليسَ المُهم ما كُنتَ بل مَا ستكون
@@ -16672,19 +16650,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B772" t="inlineStr">
+      <c r="B771" t="inlineStr">
         <is>
           <t>images/「大事なのは何者だったかじゃない。何者_img1.jpg</t>
         </is>
       </c>
-      <c r="C772" t="inlineStr">
+      <c r="C771" t="inlineStr">
         <is>
           <t>自己実現 ,存在価値</t>
         </is>
       </c>
     </row>
-    <row r="773">
-      <c r="A773" t="inlineStr">
+    <row r="772">
+      <c r="A772" t="inlineStr">
         <is>
           <t xml:space="preserve">「あなたであれ。ありのままが美しいから」
 كُنْ أَنْتَ لأنك جميل كما أنت
@@ -16693,19 +16671,19 @@
 2308 IDREES DESIGN </t>
         </is>
       </c>
-      <c r="B773" t="inlineStr">
+      <c r="B772" t="inlineStr">
         <is>
           <t>images/「あなたであれ。ありのままが美しいから_img1.jpg</t>
         </is>
       </c>
-      <c r="C773" t="inlineStr">
+      <c r="C772" t="inlineStr">
         <is>
           <t>自己肯定 ,BeYourself</t>
         </is>
       </c>
     </row>
-    <row r="774">
-      <c r="A774" t="inlineStr">
+    <row r="773">
+      <c r="A773" t="inlineStr">
         <is>
           <t xml:space="preserve">「恐れの中に生きる者は決して自由になれない」
 من يعش في خوف لن يكون حرا أبدا
@@ -16714,19 +16692,19 @@
 2111 rjeem com </t>
         </is>
       </c>
-      <c r="B774" t="inlineStr">
+      <c r="B773" t="inlineStr">
         <is>
           <t>images/「恐れの中に生きる者は決して自由になれ_img1.jpg,images/ 「恐れの中に生きる者は決して自由になれ_img2.jpg</t>
         </is>
       </c>
-      <c r="C774" t="inlineStr">
+      <c r="C773" t="inlineStr">
         <is>
           <t>勇気 ,壁</t>
         </is>
       </c>
     </row>
-    <row r="775">
-      <c r="A775" t="inlineStr">
+    <row r="774">
+      <c r="A774" t="inlineStr">
         <is>
           <t xml:space="preserve">「己の翼を信じる者は己の重さを案じない」
 من يثق في جناحيه لن يهتم لوزنه
@@ -16735,19 +16713,19 @@
 2308 kmrghani </t>
         </is>
       </c>
-      <c r="B775" t="inlineStr">
+      <c r="B774" t="inlineStr">
         <is>
           <t>images/「己の翼を信じる者は己の重さを案じない_img1.jpg</t>
         </is>
       </c>
-      <c r="C775" t="inlineStr">
+      <c r="C774" t="inlineStr">
         <is>
           <t>自信</t>
         </is>
       </c>
     </row>
-    <row r="776">
-      <c r="A776" t="inlineStr">
+    <row r="775">
+      <c r="A775" t="inlineStr">
         <is>
           <t xml:space="preserve">「珈琲で一番大事な事！誰と飲むか？」
 الأهم من القهوة!! من ستشربها معه؟
@@ -16756,19 +16734,19 @@
 1812 gwid3.tumblr </t>
         </is>
       </c>
-      <c r="B776" t="inlineStr">
+      <c r="B775" t="inlineStr">
         <is>
           <t>images/「珈琲で一番大事な事！誰と飲むか？」_img1.jpg</t>
         </is>
       </c>
-      <c r="C776" t="inlineStr">
+      <c r="C775" t="inlineStr">
         <is>
           <t>コーヒー ,名言</t>
         </is>
       </c>
     </row>
-    <row r="777">
-      <c r="A777" t="inlineStr">
+    <row r="776">
+      <c r="A776" t="inlineStr">
         <is>
           <t xml:space="preserve">「人生は美しい、そう望んだ者には。」
 الحياة جَميلَة .. لمن أراد ذلك
@@ -16778,19 +16756,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B777" t="inlineStr">
+      <c r="B776" t="inlineStr">
         <is>
           <t>images/「人生は美しい、そう望んだ者には。」_img1.jpg</t>
         </is>
       </c>
-      <c r="C777" t="inlineStr">
+      <c r="C776" t="inlineStr">
         <is>
           <t>名言 ,アート</t>
         </is>
       </c>
     </row>
-    <row r="778">
-      <c r="A778" t="inlineStr">
+    <row r="777">
+      <c r="A777" t="inlineStr">
         <is>
           <t xml:space="preserve">「ハム太郎って子を知ってるかい」
 هل تعرفون من هو هامتارو
@@ -16800,19 +16778,19 @@
 2109 </t>
         </is>
       </c>
-      <c r="B778" t="inlineStr">
+      <c r="B777" t="inlineStr">
         <is>
           <t>images/「ハム太郎って子を知ってるかい」_img1.jpg</t>
         </is>
       </c>
-      <c r="C778" t="inlineStr">
+      <c r="C777" t="inlineStr">
         <is>
           <t>オープニング ,ハム太郎</t>
         </is>
       </c>
     </row>
-    <row r="779">
-      <c r="A779" t="inlineStr">
+    <row r="778">
+      <c r="A778" t="inlineStr">
         <is>
           <t xml:space="preserve">「幸せを求める人もいれば、作る人もいる」
 هناك من يبحث عن السعادة وهناك من يصنعها
@@ -16821,19 +16799,19 @@
 2308 hindah tumblr </t>
         </is>
       </c>
-      <c r="B779" t="inlineStr">
+      <c r="B778" t="inlineStr">
         <is>
           <t>images/「幸せを求める人もいれば、作る人もいる_img1.jpg</t>
         </is>
       </c>
-      <c r="C779" t="inlineStr">
+      <c r="C778" t="inlineStr">
         <is>
           <t>幸せ ,名言 ,教訓</t>
         </is>
       </c>
     </row>
-    <row r="780">
-      <c r="A780" t="inlineStr">
+    <row r="779">
+      <c r="A779" t="inlineStr">
         <is>
           <t xml:space="preserve">「明白なるアラブの言葉によって」
 بلسان عربي مبين
@@ -16843,19 +16821,19 @@
 2109 Abdullah Barakat behance </t>
         </is>
       </c>
-      <c r="B780" t="inlineStr">
+      <c r="B779" t="inlineStr">
         <is>
           <t>images/「明白なるアラブの言葉によって」_img1.jpg</t>
         </is>
       </c>
-      <c r="C780" t="inlineStr">
+      <c r="C779" t="inlineStr">
         <is>
           <t>イスラム教 ,神聖</t>
         </is>
       </c>
     </row>
-    <row r="781">
-      <c r="A781" t="inlineStr">
+    <row r="780">
+      <c r="A780" t="inlineStr">
         <is>
           <t xml:space="preserve">「結婚前、結婚後」
 قبل الزواج، بعد الزواج
@@ -16865,19 +16843,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B781" t="inlineStr">
+      <c r="B780" t="inlineStr">
         <is>
           <t>images/「結婚前、結婚後」_img1.jpg</t>
         </is>
       </c>
-      <c r="C781" t="inlineStr">
+      <c r="C780" t="inlineStr">
         <is>
           <t>BeforeAfter ,幸せ太り</t>
         </is>
       </c>
     </row>
-    <row r="782">
-      <c r="A782" t="inlineStr">
+    <row r="781">
+      <c r="A781" t="inlineStr">
         <is>
           <t xml:space="preserve">「驚きの価格で」بسعر رائع
 ビスィアル・ラーイア [bi-si*r raa'i*]
@@ -16886,19 +16864,19 @@
 2109 Jarir Bookstore </t>
         </is>
       </c>
-      <c r="B782" t="inlineStr">
+      <c r="B781" t="inlineStr">
         <is>
           <t>images/「驚きの価格で」_img1.jpg</t>
         </is>
       </c>
-      <c r="C782" t="inlineStr">
+      <c r="C781" t="inlineStr">
         <is>
           <t>広告 ,安値</t>
         </is>
       </c>
     </row>
-    <row r="783">
-      <c r="A783" t="inlineStr">
+    <row r="782">
+      <c r="A782" t="inlineStr">
         <is>
           <t xml:space="preserve">「我が魂と共に」مع نفسي
 マア・ナフスィ [ma*a nafs-iy]
@@ -16907,19 +16885,19 @@
 2110 出典不明 </t>
         </is>
       </c>
-      <c r="B783" t="inlineStr">
+      <c r="B782" t="inlineStr">
         <is>
           <t>images/「我が魂と共に」_img1.jpg</t>
         </is>
       </c>
-      <c r="C783" t="inlineStr">
+      <c r="C782" t="inlineStr">
         <is>
           <t>ソウル ,soul</t>
         </is>
       </c>
     </row>
-    <row r="784">
-      <c r="A784" t="inlineStr">
+    <row r="783">
+      <c r="A783" t="inlineStr">
         <is>
           <t xml:space="preserve">「暗い夜に」في ليلة مظلمة
  [fiy layla(tin) mu_Dhlima(tin)]
@@ -16928,19 +16906,19 @@
 2109 سلسلة الحلزونة </t>
         </is>
       </c>
-      <c r="B784" t="inlineStr">
+      <c r="B783" t="inlineStr">
         <is>
           <t>images/「暗い夜に」_img1.jpg</t>
         </is>
       </c>
-      <c r="C784" t="inlineStr">
+      <c r="C783" t="inlineStr">
         <is>
           <t>絵本</t>
         </is>
       </c>
     </row>
-    <row r="785">
-      <c r="A785" t="inlineStr">
+    <row r="784">
+      <c r="A784" t="inlineStr">
         <is>
           <t xml:space="preserve">「ゆっくりと」بشويش
 ビシワェーシ [bi-ShwySh]
@@ -16948,19 +16926,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B785" t="inlineStr">
+      <c r="B784" t="inlineStr">
         <is>
           <t>images/「ゆっくりと」_img1.jpg</t>
         </is>
       </c>
-      <c r="C785" t="inlineStr">
+      <c r="C784" t="inlineStr">
         <is>
           <t>丸 ,円</t>
         </is>
       </c>
     </row>
-    <row r="786">
-      <c r="A786" t="inlineStr">
+    <row r="785">
+      <c r="A785" t="inlineStr">
         <is>
           <t xml:space="preserve">「この広い宇宙に…」
 في الكون الفسيح
@@ -16969,19 +16947,19 @@
 2308 wattpad </t>
         </is>
       </c>
-      <c r="B786" t="inlineStr">
+      <c r="B785" t="inlineStr">
         <is>
           <t>images/「この広い宇宙に…」_img1.jpg</t>
         </is>
       </c>
-      <c r="C786" t="inlineStr">
+      <c r="C785" t="inlineStr">
         <is>
           <t>アニメ ,宇宙</t>
         </is>
       </c>
     </row>
-    <row r="787">
-      <c r="A787" t="inlineStr">
+    <row r="786">
+      <c r="A786" t="inlineStr">
         <is>
           <t xml:space="preserve">「がんばって！」بالتوفيق
 ビッタウフィーク [bi^tawfiiq]
@@ -16989,19 +16967,19 @@
 2111 https://sites.google.com/site/mathmatic1905/ </t>
         </is>
       </c>
-      <c r="B787" t="inlineStr">
+      <c r="B786" t="inlineStr">
         <is>
           <t>images/「がんばって！」_img1.jpg</t>
         </is>
       </c>
-      <c r="C787" t="inlineStr">
+      <c r="C786" t="inlineStr">
         <is>
           <t>アラビア語</t>
         </is>
       </c>
     </row>
-    <row r="788">
-      <c r="A788" t="inlineStr">
+    <row r="787">
+      <c r="A787" t="inlineStr">
         <is>
           <t xml:space="preserve">「インターステラー」بين النجوم
 バイナ_ンヌジューム [bayna ^nujuum]
@@ -17009,19 +16987,19 @@
 2308 kmrghani </t>
         </is>
       </c>
-      <c r="B788" t="inlineStr">
+      <c r="B787" t="inlineStr">
         <is>
           <t>images/「インターステラー」_img1.jpg</t>
         </is>
       </c>
-      <c r="C788" t="inlineStr">
+      <c r="C787" t="inlineStr">
         <is>
           <t>映画 ,宇宙</t>
         </is>
       </c>
     </row>
-    <row r="789">
-      <c r="A789" t="inlineStr">
+    <row r="788">
+      <c r="A788" t="inlineStr">
         <is>
           <t xml:space="preserve">「アラビア語で」بالعربية
 ビ_ルアラビーヤ [bi-l-*arabiyya]
@@ -17030,19 +17008,19 @@
 1811 </t>
         </is>
       </c>
-      <c r="B789" t="inlineStr">
+      <c r="B788" t="inlineStr">
         <is>
           <t>images/「アラビア語で」_img1.jpg</t>
         </is>
       </c>
-      <c r="C789" t="inlineStr">
+      <c r="C788" t="inlineStr">
         <is>
           <t>ニュース ,CNN</t>
         </is>
       </c>
     </row>
-    <row r="790">
-      <c r="A790" t="inlineStr">
+    <row r="789">
+      <c r="A789" t="inlineStr">
         <is>
           <t xml:space="preserve">「17世紀に発明されて以来…」
 منذ اختراعه بالقرن السابع عشر
@@ -17050,19 +17028,19 @@
 2308 https://twitter.com/SciTalk2U/status/1450888395815854080 </t>
         </is>
       </c>
-      <c r="B790" t="inlineStr">
+      <c r="B789" t="inlineStr">
         <is>
           <t>images/「17世紀に発明されて以来…」_img1.jpg</t>
         </is>
       </c>
-      <c r="C790" t="inlineStr">
+      <c r="C789" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,望遠鏡</t>
         </is>
       </c>
     </row>
-    <row r="791">
-      <c r="A791" t="inlineStr">
+    <row r="790">
+      <c r="A790" t="inlineStr">
         <is>
           <t xml:space="preserve">「私できるよ」إنّني أستطيع
 インナニー・アスタティーウ ['inna-niy 'a-sta_tii*u]
@@ -17071,19 +17049,19 @@
 2412 سلسلة الحلزونة </t>
         </is>
       </c>
-      <c r="B791" t="inlineStr">
+      <c r="B790" t="inlineStr">
         <is>
           <t>images/「私できるよ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C791" t="inlineStr">
+      <c r="C790" t="inlineStr">
         <is>
           <t>絵本 ,こども</t>
         </is>
       </c>
     </row>
-    <row r="792">
-      <c r="A792" t="inlineStr">
+    <row r="791">
+      <c r="A791" t="inlineStr">
         <is>
           <t xml:space="preserve">「問題なし」مافيش مشكلة
 マフィーシムシュキラ [ma-fy-Sh muShkila]
@@ -17092,19 +17070,19 @@
 2109 tanzerin.theshop </t>
         </is>
       </c>
-      <c r="B792" t="inlineStr">
+      <c r="B791" t="inlineStr">
         <is>
           <t>images/「問題なし」_img1.jpg</t>
         </is>
       </c>
-      <c r="C792" t="inlineStr">
+      <c r="C791" t="inlineStr">
         <is>
           <t>シャツ ,キッズ</t>
         </is>
       </c>
     </row>
-    <row r="793">
-      <c r="A793" t="inlineStr">
+    <row r="792">
+      <c r="A792" t="inlineStr">
         <is>
           <t xml:space="preserve">「不可能はない」مفيش مستحيل
 マフィーシ・ムスタヒール [ma-fy-Sh mustaHiil]
@@ -17113,19 +17091,19 @@
 2109 أموج </t>
         </is>
       </c>
-      <c r="B793" t="inlineStr">
+      <c r="B792" t="inlineStr">
         <is>
           <t>images/「不可能はない」_img1.jpg</t>
         </is>
       </c>
-      <c r="C793" t="inlineStr">
+      <c r="C792" t="inlineStr">
         <is>
           <t>ポジティブ ,挑戦</t>
         </is>
       </c>
     </row>
-    <row r="794">
-      <c r="A794" t="inlineStr">
+    <row r="793">
+      <c r="A793" t="inlineStr">
         <is>
           <t xml:space="preserve">「等々」إلخ
 イラク ['ilaKh]
@@ -17134,19 +17112,19 @@
 2201 出典不明 </t>
         </is>
       </c>
-      <c r="B794" t="inlineStr">
+      <c r="B793" t="inlineStr">
         <is>
           <t>images/「等々」_img1.jpg</t>
         </is>
       </c>
-      <c r="C794" t="inlineStr">
+      <c r="C793" t="inlineStr">
         <is>
           <t>etc ,とんち</t>
         </is>
       </c>
     </row>
-    <row r="795">
-      <c r="A795" t="inlineStr">
+    <row r="794">
+      <c r="A794" t="inlineStr">
         <is>
           <t xml:space="preserve">⁦「調子どう？」⁩شلونَك؟
 シュローナク？ [Sh-loon-ak?]
@@ -17155,19 +17133,19 @@
 2202 Jozoor Team. </t>
         </is>
       </c>
-      <c r="B795" t="inlineStr">
+      <c r="B794" t="inlineStr">
         <is>
           <t>images/⁦「調子どう？」⁩_img1.jpg</t>
         </is>
       </c>
-      <c r="C795" t="inlineStr">
+      <c r="C794" t="inlineStr">
         <is>
           <t>洒落 ,ルービックキューブ</t>
         </is>
       </c>
     </row>
-    <row r="796">
-      <c r="A796" t="inlineStr">
+    <row r="795">
+      <c r="A795" t="inlineStr">
         <is>
           <t xml:space="preserve">「行くな」ماتروحش
 マトロホシ [ma-troH-Sh]
@@ -17176,19 +17154,19 @@
 2411 triiq tumblr </t>
         </is>
       </c>
-      <c r="B796" t="inlineStr">
+      <c r="B795" t="inlineStr">
         <is>
           <t>images/「行くな」_img1.jpg</t>
         </is>
       </c>
-      <c r="C796" t="inlineStr">
+      <c r="C795" t="inlineStr">
         <is>
           <t>ロゴ ,デザイン ,嵐</t>
         </is>
       </c>
     </row>
-    <row r="797">
-      <c r="A797" t="inlineStr">
+    <row r="796">
+      <c r="A796" t="inlineStr">
         <is>
           <t xml:space="preserve">⁦「元気？」⁩شلونَك؟
 シュローナク？ [Sh-loon-ak?]
@@ -17199,19 +17177,19 @@
 2202 出典不明 </t>
         </is>
       </c>
-      <c r="B797" t="inlineStr">
+      <c r="B796" t="inlineStr">
         <is>
           <t>images/⁦「元気？」⁩_img1.jpg</t>
         </is>
       </c>
-      <c r="C797" t="inlineStr">
+      <c r="C796" t="inlineStr">
         <is>
           <t>洒落 ,挨拶</t>
         </is>
       </c>
     </row>
-    <row r="798">
-      <c r="A798" t="inlineStr">
+    <row r="797">
+      <c r="A797" t="inlineStr">
         <is>
           <t xml:space="preserve">「気分が良いぞう」I فيل GOOD
 アイ・フィール・グッド [ai fiyl gud]
@@ -17220,19 +17198,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B798" t="inlineStr">
+      <c r="B797" t="inlineStr">
         <is>
           <t>images/「気分が良いぞう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C798" t="inlineStr">
+      <c r="C797" t="inlineStr">
         <is>
           <t>洒落 ,和訳</t>
         </is>
       </c>
     </row>
-    <row r="799">
-      <c r="A799" t="inlineStr">
+    <row r="798">
+      <c r="A798" t="inlineStr">
         <is>
           <t xml:space="preserve">「レットイットゴー／let it go」
 ليت اِت غو
@@ -17241,19 +17219,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B799" t="inlineStr">
+      <c r="B798" t="inlineStr">
         <is>
           <t>images/「レットイットゴー／let it go_img1.jpg</t>
         </is>
       </c>
-      <c r="C799" t="inlineStr">
+      <c r="C798" t="inlineStr">
         <is>
           <t>折衷 ,アナ雪</t>
         </is>
       </c>
     </row>
-    <row r="800">
-      <c r="A800" t="inlineStr">
+    <row r="799">
+      <c r="A799" t="inlineStr">
         <is>
           <t xml:space="preserve">「ようこそ」اهلا وسهلا
 アハラン・ワサハラン ['ahlan wa-sahlan]
@@ -17261,19 +17239,19 @@
 2106 behance Anwar Al Eissa </t>
         </is>
       </c>
-      <c r="B800" t="inlineStr">
+      <c r="B799" t="inlineStr">
         <is>
           <t>images/「ようこそ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C800" t="inlineStr">
+      <c r="C799" t="inlineStr">
         <is>
           <t>アラビア語</t>
         </is>
       </c>
     </row>
-    <row r="801">
-      <c r="A801" t="inlineStr">
+    <row r="800">
+      <c r="A800" t="inlineStr">
         <is>
           <t xml:space="preserve">「まぁ何というサプライズでしょう」
 يا لها من مفاجأة
@@ -17284,19 +17262,19 @@
 2108 neelwafurat com </t>
         </is>
       </c>
-      <c r="B801" t="inlineStr">
+      <c r="B800" t="inlineStr">
         <is>
           <t>images/「まぁ何というサプライズでしょう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C801" t="inlineStr">
+      <c r="C800" t="inlineStr">
         <is>
           <t>中国語 ,学習</t>
         </is>
       </c>
     </row>
-    <row r="802">
-      <c r="A802" t="inlineStr">
+    <row r="801">
+      <c r="A801" t="inlineStr">
         <is>
           <t xml:space="preserve">「ハックション」اتشوو
 アチュー！ ['aatShuu]
@@ -17304,19 +17282,19 @@
 1811 </t>
         </is>
       </c>
-      <c r="B802" t="inlineStr">
+      <c r="B801" t="inlineStr">
         <is>
           <t>images/「ハックション」_img1.jpg</t>
         </is>
       </c>
-      <c r="C802" t="inlineStr">
+      <c r="C801" t="inlineStr">
         <is>
           <t>あらびあや</t>
         </is>
       </c>
     </row>
-    <row r="803">
-      <c r="A803" t="inlineStr">
+    <row r="802">
+      <c r="A802" t="inlineStr">
         <is>
           <t xml:space="preserve">「スブハーナッラー」「アルハムドゥリッラー」「アッラーアクバル」
 سبحان الله
@@ -17327,19 +17305,19 @@
 2308 dribbble com </t>
         </is>
       </c>
-      <c r="B803" t="inlineStr">
+      <c r="B802" t="inlineStr">
         <is>
           <t>images/「スブハーナッラー」「アルハムドゥリッ_img1.jpg</t>
         </is>
       </c>
-      <c r="C803" t="inlineStr">
+      <c r="C802" t="inlineStr">
         <is>
           <t>四角 ,コンパクト</t>
         </is>
       </c>
     </row>
-    <row r="804">
-      <c r="A804" t="inlineStr">
+    <row r="803">
+      <c r="A803" t="inlineStr">
         <is>
           <t xml:space="preserve">「すごく美味しい！」لذيذ جدًا
 ラズィーズ・ジッダン [laDhiiDh jiddan]
@@ -17348,19 +17326,19 @@
 2109 goodreads com </t>
         </is>
       </c>
-      <c r="B804" t="inlineStr">
+      <c r="B803" t="inlineStr">
         <is>
           <t>images/「すごく美味しい！」_img1.jpg</t>
         </is>
       </c>
-      <c r="C804" t="inlineStr">
+      <c r="C803" t="inlineStr">
         <is>
           <t>フレーズ ,感想</t>
         </is>
       </c>
     </row>
-    <row r="805">
-      <c r="A805" t="inlineStr">
+    <row r="804">
+      <c r="A804" t="inlineStr">
         <is>
           <t xml:space="preserve">「しとしと、雨」تك تك يا مطر
 ティクティク [tik tik yaa ma_tar]
@@ -17369,19 +17347,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B805" t="inlineStr">
+      <c r="B804" t="inlineStr">
         <is>
           <t>images/「しとしと、雨」_img1.jpg</t>
         </is>
       </c>
-      <c r="C805" t="inlineStr">
+      <c r="C804" t="inlineStr">
         <is>
           <t>天気 ,梅雨</t>
         </is>
       </c>
     </row>
-    <row r="806">
-      <c r="A806" t="inlineStr">
+    <row r="805">
+      <c r="A805" t="inlineStr">
         <is>
           <t xml:space="preserve">「さかさま」رأساً على عقب
 ラッアサン・アラー・アケブ [ra'san *alaa *aqib]
@@ -17389,19 +17367,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B806" t="inlineStr">
+      <c r="B805" t="inlineStr">
         <is>
           <t>images/「さかさま」_img1.jpg</t>
         </is>
       </c>
-      <c r="C806" t="inlineStr">
+      <c r="C805" t="inlineStr">
         <is>
           <t>壁 ,上下</t>
         </is>
       </c>
     </row>
-    <row r="807">
-      <c r="A807" t="inlineStr">
+    <row r="806">
+      <c r="A806" t="inlineStr">
         <is>
           <t xml:space="preserve">「エジプトよどこへ行った」
 فينك يا مصر؟
@@ -17411,19 +17389,19 @@
 1809 shehabfawzy1.tumblr </t>
         </is>
       </c>
-      <c r="B807" t="inlineStr">
+      <c r="B806" t="inlineStr">
         <is>
           <t>images/「エジプトよどこへ行った」_img1.jpg</t>
         </is>
       </c>
-      <c r="C807" t="inlineStr">
+      <c r="C806" t="inlineStr">
         <is>
           <t>ピラミッド ,歴史</t>
         </is>
       </c>
     </row>
-    <row r="808">
-      <c r="A808" t="inlineStr">
+    <row r="807">
+      <c r="A807" t="inlineStr">
         <is>
           <t xml:space="preserve">「ありがとう」شكراً
 シュクラン [Shukran]
@@ -17431,19 +17409,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B808" t="inlineStr">
+      <c r="B807" t="inlineStr">
         <is>
           <t>images/「ありがとう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C808" t="inlineStr">
+      <c r="C807" t="inlineStr">
         <is>
           <t>挨拶 ,文字</t>
         </is>
       </c>
     </row>
-    <row r="809">
-      <c r="A809" t="inlineStr">
+    <row r="808">
+      <c r="A808" t="inlineStr">
         <is>
           <t xml:space="preserve">「昼寝の時間だ」
 إنه وقت القيلولة
@@ -17452,12 +17430,12 @@
 2501 https://x.com/NatGeoMagArab/status/1858049951579910486 </t>
         </is>
       </c>
-      <c r="B809" t="inlineStr">
+      <c r="B808" t="inlineStr">
         <is>
           <t>images/「昼寝の時間だ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C809" t="inlineStr">
+      <c r="C808" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,ペンギン</t>
         </is>

</xml_diff>